<commit_message>
Adicionar modulo de servico na base de dados
</commit_message>
<xml_diff>
--- a/base de dados.xlsx
+++ b/base de dados.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesle\Documents\Projeto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesle\Desktop\Projeto-Power-BI-Oficina-Mecanica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{333685CC-ECE8-4D7E-A14E-EEF04B7A742A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C146922-ABDD-4354-9730-FB5D9F119A36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11640" activeTab="1" xr2:uid="{C68C1244-3D4F-43FC-8114-B501E2A75E8B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11640" activeTab="2" xr2:uid="{C68C1244-3D4F-43FC-8114-B501E2A75E8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Cliente" sheetId="1" r:id="rId1"/>
     <sheet name="Tabela  Serviços" sheetId="2" r:id="rId2"/>
+    <sheet name="Ordens de Serviço" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>ID_Cliente</t>
   </si>
@@ -103,6 +104,21 @@
   </si>
   <si>
     <t>Revisao geral</t>
+  </si>
+  <si>
+    <t>ID_OS</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Quantidade</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 10/01/2026 </t>
   </si>
 </sst>
 </file>
@@ -138,8 +154,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -631,4 +648,237 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43212B5B-FBAB-4DDC-989A-2A4BDF07DDD2}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>46023</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46024</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46027</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>46037</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1">
+        <v>46042</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1">
+        <v>46047</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1">
+        <v>46054</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1">
+        <v>46056</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1">
+        <v>46058</v>
+      </c>
+      <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
editando base de dados texto
</commit_message>
<xml_diff>
--- a/base de dados.xlsx
+++ b/base de dados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesle\Desktop\Projeto-Power-BI-Oficina-Mecanica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA0B251-87D9-40D4-8027-E218C694B4E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86451E4A-036F-4F8D-B32A-0D6D87CE1E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11640" activeTab="1" xr2:uid="{C68C1244-3D4F-43FC-8114-B501E2A75E8B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11640" xr2:uid="{C68C1244-3D4F-43FC-8114-B501E2A75E8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Cliente" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="171">
   <si>
     <t>ID_Cliente</t>
   </si>
@@ -49,36 +49,12 @@
     <t>Nome</t>
   </si>
   <si>
-    <t>João Silva</t>
-  </si>
-  <si>
-    <t>Maria Souza</t>
-  </si>
-  <si>
-    <t>Carlos Lima</t>
-  </si>
-  <si>
-    <t>Ana Pereira</t>
-  </si>
-  <si>
-    <t>Roberto Costa</t>
-  </si>
-  <si>
     <t>São Paulo</t>
   </si>
   <si>
     <t>Cidade</t>
   </si>
   <si>
-    <t>Osasco</t>
-  </si>
-  <si>
-    <t>Santo André</t>
-  </si>
-  <si>
-    <t>São Bernardo</t>
-  </si>
-  <si>
     <t>ID_Serviço</t>
   </si>
   <si>
@@ -116,6 +92,468 @@
   </si>
   <si>
     <t xml:space="preserve"> 10/01/2026 </t>
+  </si>
+  <si>
+    <t>Lucas</t>
+  </si>
+  <si>
+    <t>Ana</t>
+  </si>
+  <si>
+    <t>Pedro</t>
+  </si>
+  <si>
+    <t>Mariana</t>
+  </si>
+  <si>
+    <t>João</t>
+  </si>
+  <si>
+    <t>Juliana</t>
+  </si>
+  <si>
+    <t>Gabriel</t>
+  </si>
+  <si>
+    <t>Camila</t>
+  </si>
+  <si>
+    <t>Rafael</t>
+  </si>
+  <si>
+    <t>Larissa</t>
+  </si>
+  <si>
+    <t>Bruno</t>
+  </si>
+  <si>
+    <t>Fernanda</t>
+  </si>
+  <si>
+    <t>Carlos</t>
+  </si>
+  <si>
+    <t>Beatriz</t>
+  </si>
+  <si>
+    <t>Diego</t>
+  </si>
+  <si>
+    <t>Amanda</t>
+  </si>
+  <si>
+    <t>Felipe</t>
+  </si>
+  <si>
+    <t>Aline</t>
+  </si>
+  <si>
+    <t>Rodrigo</t>
+  </si>
+  <si>
+    <t>Patrícia</t>
+  </si>
+  <si>
+    <t>Gustavo</t>
+  </si>
+  <si>
+    <t>Bianca</t>
+  </si>
+  <si>
+    <t>Eduardo</t>
+  </si>
+  <si>
+    <t>Daniela</t>
+  </si>
+  <si>
+    <t>Vinícius</t>
+  </si>
+  <si>
+    <t>Renata</t>
+  </si>
+  <si>
+    <t>Matheus</t>
+  </si>
+  <si>
+    <t>Carla</t>
+  </si>
+  <si>
+    <t>André</t>
+  </si>
+  <si>
+    <t>Priscila</t>
+  </si>
+  <si>
+    <t>Leonardo</t>
+  </si>
+  <si>
+    <t>Vanessa</t>
+  </si>
+  <si>
+    <t>Henrique</t>
+  </si>
+  <si>
+    <t>Débora</t>
+  </si>
+  <si>
+    <t>Marcelo</t>
+  </si>
+  <si>
+    <t>Letícia</t>
+  </si>
+  <si>
+    <t>Tiago</t>
+  </si>
+  <si>
+    <t>Natália</t>
+  </si>
+  <si>
+    <t>Daniel</t>
+  </si>
+  <si>
+    <t>Rafaela</t>
+  </si>
+  <si>
+    <t>Alexandre</t>
+  </si>
+  <si>
+    <t>Tatiane</t>
+  </si>
+  <si>
+    <t>César</t>
+  </si>
+  <si>
+    <t>Elaine</t>
+  </si>
+  <si>
+    <t>Fábio</t>
+  </si>
+  <si>
+    <t>Sandra</t>
+  </si>
+  <si>
+    <t>Sérgio</t>
+  </si>
+  <si>
+    <t>Rosana</t>
+  </si>
+  <si>
+    <t>Paulo</t>
+  </si>
+  <si>
+    <t>Cláudia</t>
+  </si>
+  <si>
+    <t>Jorge</t>
+  </si>
+  <si>
+    <t>Márcia</t>
+  </si>
+  <si>
+    <t>Renato</t>
+  </si>
+  <si>
+    <t>Silvia</t>
+  </si>
+  <si>
+    <t>Otávio</t>
+  </si>
+  <si>
+    <t>Adriana</t>
+  </si>
+  <si>
+    <t>Igor</t>
+  </si>
+  <si>
+    <t>Lúcia</t>
+  </si>
+  <si>
+    <t>Caio</t>
+  </si>
+  <si>
+    <t>Suellen</t>
+  </si>
+  <si>
+    <t>Victor</t>
+  </si>
+  <si>
+    <t>Mirela</t>
+  </si>
+  <si>
+    <t>Wesley</t>
+  </si>
+  <si>
+    <t>Jéssica</t>
+  </si>
+  <si>
+    <t>Alan</t>
+  </si>
+  <si>
+    <t>Kelly</t>
+  </si>
+  <si>
+    <t>Denis</t>
+  </si>
+  <si>
+    <t>Cristiane</t>
+  </si>
+  <si>
+    <t>Hugo</t>
+  </si>
+  <si>
+    <t>Flávia</t>
+  </si>
+  <si>
+    <t>Yuri</t>
+  </si>
+  <si>
+    <t>Roberta</t>
+  </si>
+  <si>
+    <t>Davi</t>
+  </si>
+  <si>
+    <t>Elisângela</t>
+  </si>
+  <si>
+    <t>Murilo</t>
+  </si>
+  <si>
+    <t>Cíntia</t>
+  </si>
+  <si>
+    <t>Samuel</t>
+  </si>
+  <si>
+    <t>Josiane</t>
+  </si>
+  <si>
+    <t>Elias</t>
+  </si>
+  <si>
+    <t>Jaqueline</t>
+  </si>
+  <si>
+    <t>Joel</t>
+  </si>
+  <si>
+    <t>Franciele</t>
+  </si>
+  <si>
+    <t>Leandro</t>
+  </si>
+  <si>
+    <t>Tatiana</t>
+  </si>
+  <si>
+    <t>Michel</t>
+  </si>
+  <si>
+    <t>Kátia</t>
+  </si>
+  <si>
+    <t>Nelson</t>
+  </si>
+  <si>
+    <t>Ivone</t>
+  </si>
+  <si>
+    <t>Ricardo</t>
+  </si>
+  <si>
+    <t>Regina</t>
+  </si>
+  <si>
+    <t>Alberto</t>
+  </si>
+  <si>
+    <t>Gisele</t>
+  </si>
+  <si>
+    <t>Cláudio</t>
+  </si>
+  <si>
+    <t>Fabiana</t>
+  </si>
+  <si>
+    <t>Valter</t>
+  </si>
+  <si>
+    <t>Bruna</t>
+  </si>
+  <si>
+    <t>Armando</t>
+  </si>
+  <si>
+    <t>Daiane</t>
+  </si>
+  <si>
+    <t>Francisco</t>
+  </si>
+  <si>
+    <t>Érica</t>
+  </si>
+  <si>
+    <t>Gilberto</t>
+  </si>
+  <si>
+    <t>Luciana</t>
+  </si>
+  <si>
+    <t>Heitor</t>
+  </si>
+  <si>
+    <t>Paula</t>
+  </si>
+  <si>
+    <t>Isaac</t>
+  </si>
+  <si>
+    <t>Sônia</t>
+  </si>
+  <si>
+    <t>Jonas</t>
+  </si>
+  <si>
+    <t>Lorena</t>
+  </si>
+  <si>
+    <t>Kevin</t>
+  </si>
+  <si>
+    <t>Milena</t>
+  </si>
+  <si>
+    <t>Luan</t>
+  </si>
+  <si>
+    <t>Yasmin</t>
+  </si>
+  <si>
+    <t>Nathan</t>
+  </si>
+  <si>
+    <t>Vitória</t>
+  </si>
+  <si>
+    <t>Oliver</t>
+  </si>
+  <si>
+    <t>Sabrina</t>
+  </si>
+  <si>
+    <t>Patrick</t>
+  </si>
+  <si>
+    <t>Tamara</t>
+  </si>
+  <si>
+    <t>Raul</t>
+  </si>
+  <si>
+    <t>Alana</t>
+  </si>
+  <si>
+    <t>Enzo</t>
+  </si>
+  <si>
+    <t>Isabela</t>
+  </si>
+  <si>
+    <t>Theo</t>
+  </si>
+  <si>
+    <t>Helena</t>
+  </si>
+  <si>
+    <t>Gael</t>
+  </si>
+  <si>
+    <t>Nicole</t>
+  </si>
+  <si>
+    <t>Bento</t>
+  </si>
+  <si>
+    <t>Alice</t>
+  </si>
+  <si>
+    <t>Pietro</t>
+  </si>
+  <si>
+    <t>Laura</t>
+  </si>
+  <si>
+    <t>Noah</t>
+  </si>
+  <si>
+    <t>Aurora</t>
+  </si>
+  <si>
+    <t>Levi</t>
+  </si>
+  <si>
+    <t>Clara</t>
+  </si>
+  <si>
+    <t>Benício</t>
+  </si>
+  <si>
+    <t>Elisa</t>
+  </si>
+  <si>
+    <t>Vicente</t>
+  </si>
+  <si>
+    <t>Lívia</t>
+  </si>
+  <si>
+    <t>Augusto</t>
+  </si>
+  <si>
+    <t>Sofia</t>
+  </si>
+  <si>
+    <t>Artur</t>
+  </si>
+  <si>
+    <t>Cecília</t>
+  </si>
+  <si>
+    <t>Joaquim</t>
+  </si>
+  <si>
+    <t>Manuella</t>
+  </si>
+  <si>
+    <t>Bernardo</t>
+  </si>
+  <si>
+    <t>Antonella</t>
+  </si>
+  <si>
+    <t>Dante</t>
+  </si>
+  <si>
+    <t>Rebeca</t>
+  </si>
+  <si>
+    <t>Tomás</t>
+  </si>
+  <si>
+    <t>Ester</t>
+  </si>
+  <si>
+    <t>Rio de Janeiro</t>
+  </si>
+  <si>
+    <t>Belo Horizonte</t>
+  </si>
+  <si>
+    <t>Salvador</t>
+  </si>
+  <si>
+    <t>Brasília</t>
   </si>
 </sst>
 </file>
@@ -488,9 +926,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47DEE4CA-CEFF-4D30-B427-5B29E0AA61DD}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C153"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
@@ -503,7 +942,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -511,10 +950,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -522,10 +961,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -533,10 +972,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -544,10 +983,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -555,10 +994,1627 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C26" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C27" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>47</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>48</v>
+      </c>
+      <c r="C33" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>49</v>
+      </c>
+      <c r="C34" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>50</v>
+      </c>
+      <c r="C35" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>51</v>
+      </c>
+      <c r="C36" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>53</v>
+      </c>
+      <c r="C38" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>54</v>
+      </c>
+      <c r="C39" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>55</v>
+      </c>
+      <c r="C40" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>56</v>
+      </c>
+      <c r="C41" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>58</v>
+      </c>
+      <c r="C43" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>59</v>
+      </c>
+      <c r="C44" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>60</v>
+      </c>
+      <c r="C45" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>61</v>
+      </c>
+      <c r="C46" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>62</v>
+      </c>
+      <c r="C47" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>63</v>
+      </c>
+      <c r="C48" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>64</v>
+      </c>
+      <c r="C49" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
+        <v>65</v>
+      </c>
+      <c r="C50" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>66</v>
+      </c>
+      <c r="C51" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>67</v>
+      </c>
+      <c r="C52" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>68</v>
+      </c>
+      <c r="C53" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>69</v>
+      </c>
+      <c r="C54" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>70</v>
+      </c>
+      <c r="C55" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>71</v>
+      </c>
+      <c r="C56" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>72</v>
+      </c>
+      <c r="C57" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>73</v>
+      </c>
+      <c r="C58" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>74</v>
+      </c>
+      <c r="C59" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>75</v>
+      </c>
+      <c r="C60" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>76</v>
+      </c>
+      <c r="C61" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>77</v>
+      </c>
+      <c r="C62" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>78</v>
+      </c>
+      <c r="C63" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>79</v>
+      </c>
+      <c r="C64" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>80</v>
+      </c>
+      <c r="C65" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>81</v>
+      </c>
+      <c r="C66" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>82</v>
+      </c>
+      <c r="C67" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>83</v>
+      </c>
+      <c r="C68" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>84</v>
+      </c>
+      <c r="C69" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>85</v>
+      </c>
+      <c r="C70" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>86</v>
+      </c>
+      <c r="C71" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>87</v>
+      </c>
+      <c r="C72" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>88</v>
+      </c>
+      <c r="C73" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>89</v>
+      </c>
+      <c r="C74" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>90</v>
+      </c>
+      <c r="C75" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>91</v>
+      </c>
+      <c r="C76" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>92</v>
+      </c>
+      <c r="C77" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>93</v>
+      </c>
+      <c r="C78" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>94</v>
+      </c>
+      <c r="C79" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>95</v>
+      </c>
+      <c r="C80" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>96</v>
+      </c>
+      <c r="C81" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>97</v>
+      </c>
+      <c r="C82" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>98</v>
+      </c>
+      <c r="C83" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>99</v>
+      </c>
+      <c r="C84" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>100</v>
+      </c>
+      <c r="C85" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
+        <v>101</v>
+      </c>
+      <c r="C86" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>102</v>
+      </c>
+      <c r="C87" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>103</v>
+      </c>
+      <c r="C88" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>104</v>
+      </c>
+      <c r="C89" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>105</v>
+      </c>
+      <c r="C90" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
+        <v>106</v>
+      </c>
+      <c r="C91" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
+        <v>107</v>
+      </c>
+      <c r="C92" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>108</v>
+      </c>
+      <c r="C93" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>109</v>
+      </c>
+      <c r="C94" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>110</v>
+      </c>
+      <c r="C95" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="s">
+        <v>111</v>
+      </c>
+      <c r="C96" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>112</v>
+      </c>
+      <c r="C97" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
+        <v>113</v>
+      </c>
+      <c r="C98" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="s">
+        <v>114</v>
+      </c>
+      <c r="C99" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="s">
+        <v>115</v>
+      </c>
+      <c r="C100" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" t="s">
+        <v>116</v>
+      </c>
+      <c r="C101" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102" t="s">
+        <v>117</v>
+      </c>
+      <c r="C102" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103" t="s">
+        <v>118</v>
+      </c>
+      <c r="C103" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104" t="s">
+        <v>119</v>
+      </c>
+      <c r="C104" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105" t="s">
+        <v>120</v>
+      </c>
+      <c r="C105" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106" t="s">
+        <v>121</v>
+      </c>
+      <c r="C106" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107" t="s">
+        <v>122</v>
+      </c>
+      <c r="C107" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108" t="s">
+        <v>123</v>
+      </c>
+      <c r="C108" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109" t="s">
+        <v>124</v>
+      </c>
+      <c r="C109" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110" t="s">
+        <v>125</v>
+      </c>
+      <c r="C110" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111" t="s">
+        <v>126</v>
+      </c>
+      <c r="C111" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112" t="s">
+        <v>127</v>
+      </c>
+      <c r="C112" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113" t="s">
+        <v>128</v>
+      </c>
+      <c r="C113" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>113</v>
+      </c>
+      <c r="B114" t="s">
+        <v>129</v>
+      </c>
+      <c r="C114" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115" t="s">
+        <v>130</v>
+      </c>
+      <c r="C115" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116" t="s">
+        <v>131</v>
+      </c>
+      <c r="C116" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117" t="s">
+        <v>132</v>
+      </c>
+      <c r="C117" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118" t="s">
+        <v>133</v>
+      </c>
+      <c r="C118" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119" t="s">
+        <v>134</v>
+      </c>
+      <c r="C119" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120" t="s">
+        <v>135</v>
+      </c>
+      <c r="C120" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121" t="s">
+        <v>136</v>
+      </c>
+      <c r="C121" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>121</v>
+      </c>
+      <c r="B122" t="s">
+        <v>137</v>
+      </c>
+      <c r="C122" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>122</v>
+      </c>
+      <c r="B123" t="s">
+        <v>138</v>
+      </c>
+      <c r="C123" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>123</v>
+      </c>
+      <c r="B124" t="s">
+        <v>139</v>
+      </c>
+      <c r="C124" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125">
+        <v>124</v>
+      </c>
+      <c r="B125" t="s">
+        <v>140</v>
+      </c>
+      <c r="C125" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>125</v>
+      </c>
+      <c r="B126" t="s">
+        <v>141</v>
+      </c>
+      <c r="C126" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127">
+        <v>126</v>
+      </c>
+      <c r="B127" t="s">
+        <v>142</v>
+      </c>
+      <c r="C127" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128" t="s">
+        <v>143</v>
+      </c>
+      <c r="C128" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129" t="s">
+        <v>144</v>
+      </c>
+      <c r="C129" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130" t="s">
+        <v>145</v>
+      </c>
+      <c r="C130" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131" t="s">
+        <v>146</v>
+      </c>
+      <c r="C131" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132" t="s">
+        <v>147</v>
+      </c>
+      <c r="C132" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133" t="s">
+        <v>148</v>
+      </c>
+      <c r="C133" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134" t="s">
+        <v>149</v>
+      </c>
+      <c r="C134" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135" t="s">
+        <v>150</v>
+      </c>
+      <c r="C135" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136" t="s">
+        <v>151</v>
+      </c>
+      <c r="C136" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137" t="s">
+        <v>152</v>
+      </c>
+      <c r="C137" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138" t="s">
+        <v>153</v>
+      </c>
+      <c r="C138" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139" t="s">
+        <v>154</v>
+      </c>
+      <c r="C139" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140" t="s">
+        <v>155</v>
+      </c>
+      <c r="C140" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141" t="s">
+        <v>156</v>
+      </c>
+      <c r="C141" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142" t="s">
+        <v>157</v>
+      </c>
+      <c r="C142" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143">
+        <v>142</v>
+      </c>
+      <c r="B143" t="s">
+        <v>158</v>
+      </c>
+      <c r="C143" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144">
+        <v>143</v>
+      </c>
+      <c r="B144" t="s">
+        <v>159</v>
+      </c>
+      <c r="C144" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145">
+        <v>144</v>
+      </c>
+      <c r="B145" t="s">
+        <v>160</v>
+      </c>
+      <c r="C145" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146">
+        <v>145</v>
+      </c>
+      <c r="B146" t="s">
+        <v>161</v>
+      </c>
+      <c r="C146" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147">
+        <v>146</v>
+      </c>
+      <c r="B147" t="s">
+        <v>162</v>
+      </c>
+      <c r="C147" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148">
+        <v>147</v>
+      </c>
+      <c r="B148" t="s">
+        <v>163</v>
+      </c>
+      <c r="C148" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149">
+        <v>148</v>
+      </c>
+      <c r="B149" t="s">
+        <v>164</v>
+      </c>
+      <c r="C149" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150">
+        <v>149</v>
+      </c>
+      <c r="B150" t="s">
+        <v>165</v>
+      </c>
+      <c r="C150" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151">
+        <v>150</v>
+      </c>
+      <c r="B151" t="s">
+        <v>166</v>
+      </c>
+      <c r="C151" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A152">
+        <v>151</v>
+      </c>
+      <c r="B152" t="s">
+        <v>135</v>
+      </c>
+      <c r="C152" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A153">
+        <v>152</v>
+      </c>
+      <c r="B153" t="s">
+        <v>85</v>
+      </c>
+      <c r="C153" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -576,13 +2632,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -590,7 +2646,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C2">
         <v>120</v>
@@ -601,7 +2657,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C3">
         <v>80</v>
@@ -612,7 +2668,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C4">
         <v>300</v>
@@ -623,7 +2679,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C5">
         <v>450</v>
@@ -634,7 +2690,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>11</v>
+      </c>
+      <c r="C6">
+        <v>900</v>
       </c>
     </row>
   </sheetData>
@@ -648,26 +2707,27 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F1" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -735,7 +2795,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C5">
         <v>3</v>

</xml_diff>

<commit_message>
insert valor e serviço
</commit_message>
<xml_diff>
--- a/base de dados.xlsx
+++ b/base de dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesle\Desktop\Projeto-Power-BI-Oficina-Mecanica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86451E4A-036F-4F8D-B32A-0D6D87CE1E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{185D673A-788A-408E-8B03-85C8EB602BBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11640" xr2:uid="{C68C1244-3D4F-43FC-8114-B501E2A75E8B}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="173">
   <si>
     <t>ID_Cliente</t>
   </si>
@@ -554,6 +554,12 @@
   </si>
   <si>
     <t>Brasília</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor </t>
+  </si>
+  <si>
+    <t>Serviço</t>
   </si>
 </sst>
 </file>
@@ -589,9 +595,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -926,15 +935,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47DEE4CA-CEFF-4D30-B427-5B29E0AA61DD}">
-  <dimension ref="A1:C153"/>
+  <dimension ref="A1:E154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -944,8 +955,14 @@
       <c r="C1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>171</v>
+      </c>
+      <c r="E1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -955,8 +972,14 @@
       <c r="C2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <v>900</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -966,8 +989,14 @@
       <c r="C3" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D3">
+        <v>120</v>
+      </c>
+      <c r="E3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -977,8 +1006,14 @@
       <c r="C4" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <v>120</v>
+      </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -988,8 +1023,14 @@
       <c r="C5" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5">
+        <v>900</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -999,8 +1040,14 @@
       <c r="C6" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6">
+        <v>900</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1010,8 +1057,14 @@
       <c r="C7" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <v>80</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1021,8 +1074,14 @@
       <c r="C8" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D8">
+        <v>900</v>
+      </c>
+      <c r="E8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1032,8 +1091,14 @@
       <c r="C9" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <v>120</v>
+      </c>
+      <c r="E9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1043,8 +1108,14 @@
       <c r="C10" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10">
+        <v>900</v>
+      </c>
+      <c r="E10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1054,8 +1125,14 @@
       <c r="C11" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11">
+        <v>900</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1065,8 +1142,14 @@
       <c r="C12" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12">
+        <v>80</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1076,8 +1159,14 @@
       <c r="C13" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D13">
+        <v>80</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1087,8 +1176,14 @@
       <c r="C14" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D14">
+        <v>900</v>
+      </c>
+      <c r="E14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1098,8 +1193,14 @@
       <c r="C15" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D15">
+        <v>80</v>
+      </c>
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1109,8 +1210,14 @@
       <c r="C16" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D16">
+        <v>900</v>
+      </c>
+      <c r="E16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1120,8 +1227,14 @@
       <c r="C17" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D17">
+        <v>80</v>
+      </c>
+      <c r="E17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1131,8 +1244,14 @@
       <c r="C18" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D18">
+        <v>80</v>
+      </c>
+      <c r="E18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1142,8 +1261,14 @@
       <c r="C19" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19">
+        <v>900</v>
+      </c>
+      <c r="E19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1153,8 +1278,14 @@
       <c r="C20" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D20">
+        <v>80</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1164,8 +1295,14 @@
       <c r="C21" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D21">
+        <v>80</v>
+      </c>
+      <c r="E21" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1175,8 +1312,14 @@
       <c r="C22" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D22">
+        <v>900</v>
+      </c>
+      <c r="E22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1186,8 +1329,14 @@
       <c r="C23" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D23">
+        <v>900</v>
+      </c>
+      <c r="E23" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1197,8 +1346,14 @@
       <c r="C24" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D24">
+        <v>120</v>
+      </c>
+      <c r="E24" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1208,8 +1363,14 @@
       <c r="C25" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D25">
+        <v>120</v>
+      </c>
+      <c r="E25" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1219,8 +1380,14 @@
       <c r="C26" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D26">
+        <v>120</v>
+      </c>
+      <c r="E26" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1230,8 +1397,14 @@
       <c r="C27" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D27">
+        <v>120</v>
+      </c>
+      <c r="E27" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1241,8 +1414,14 @@
       <c r="C28" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D28">
+        <v>120</v>
+      </c>
+      <c r="E28" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1252,8 +1431,14 @@
       <c r="C29" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D29">
+        <v>900</v>
+      </c>
+      <c r="E29" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1263,8 +1448,14 @@
       <c r="C30" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D30">
+        <v>300</v>
+      </c>
+      <c r="E30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1274,8 +1465,14 @@
       <c r="C31" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D31">
+        <v>300</v>
+      </c>
+      <c r="E31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1285,8 +1482,14 @@
       <c r="C32" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D32">
+        <v>300</v>
+      </c>
+      <c r="E32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1296,8 +1499,14 @@
       <c r="C33" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D33">
+        <v>300</v>
+      </c>
+      <c r="E33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1307,8 +1516,14 @@
       <c r="C34" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D34">
+        <v>300</v>
+      </c>
+      <c r="E34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1318,8 +1533,14 @@
       <c r="C35" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D35">
+        <v>900</v>
+      </c>
+      <c r="E35" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1329,8 +1550,14 @@
       <c r="C36" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D36">
+        <v>450</v>
+      </c>
+      <c r="E36" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1340,8 +1567,14 @@
       <c r="C37" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D37">
+        <v>450</v>
+      </c>
+      <c r="E37" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1351,8 +1584,14 @@
       <c r="C38" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D38">
+        <v>450</v>
+      </c>
+      <c r="E38" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1362,8 +1601,14 @@
       <c r="C39" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D39">
+        <v>900</v>
+      </c>
+      <c r="E39" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1373,8 +1618,14 @@
       <c r="C40" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D40">
+        <v>450</v>
+      </c>
+      <c r="E40" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1384,8 +1635,14 @@
       <c r="C41" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D41">
+        <v>450</v>
+      </c>
+      <c r="E41" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1395,8 +1652,14 @@
       <c r="C42" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D42">
+        <v>450</v>
+      </c>
+      <c r="E42" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1406,8 +1669,14 @@
       <c r="C43" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D43">
+        <v>120</v>
+      </c>
+      <c r="E43" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1417,8 +1686,14 @@
       <c r="C44" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D44">
+        <v>120</v>
+      </c>
+      <c r="E44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1428,8 +1703,14 @@
       <c r="C45" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D45">
+        <v>120</v>
+      </c>
+      <c r="E45" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1439,8 +1720,14 @@
       <c r="C46" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D46">
+        <v>120</v>
+      </c>
+      <c r="E46" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1450,8 +1737,14 @@
       <c r="C47" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D47">
+        <v>120</v>
+      </c>
+      <c r="E47" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1461,8 +1754,14 @@
       <c r="C48" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D48">
+        <v>120</v>
+      </c>
+      <c r="E48" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1472,8 +1771,14 @@
       <c r="C49" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D49">
+        <v>450</v>
+      </c>
+      <c r="E49" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1483,8 +1788,14 @@
       <c r="C50" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D50">
+        <v>450</v>
+      </c>
+      <c r="E50" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1494,8 +1805,14 @@
       <c r="C51" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D51">
+        <v>450</v>
+      </c>
+      <c r="E51" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1505,8 +1822,14 @@
       <c r="C52" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D52">
+        <v>450</v>
+      </c>
+      <c r="E52" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1516,8 +1839,14 @@
       <c r="C53" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D53">
+        <v>900</v>
+      </c>
+      <c r="E53" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1527,8 +1856,14 @@
       <c r="C54" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D54">
+        <v>450</v>
+      </c>
+      <c r="E54" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1538,8 +1873,14 @@
       <c r="C55" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D55">
+        <v>450</v>
+      </c>
+      <c r="E55" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1549,8 +1890,14 @@
       <c r="C56" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D56">
+        <v>450</v>
+      </c>
+      <c r="E56" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1560,8 +1907,14 @@
       <c r="C57" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D57">
+        <v>450</v>
+      </c>
+      <c r="E57" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1571,8 +1924,14 @@
       <c r="C58" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D58">
+        <v>450</v>
+      </c>
+      <c r="E58" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -1582,8 +1941,14 @@
       <c r="C59" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D59">
+        <v>450</v>
+      </c>
+      <c r="E59" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -1593,8 +1958,14 @@
       <c r="C60" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D60">
+        <v>450</v>
+      </c>
+      <c r="E60" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -1604,8 +1975,14 @@
       <c r="C61" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D61">
+        <v>450</v>
+      </c>
+      <c r="E61" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -1615,8 +1992,14 @@
       <c r="C62" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D62">
+        <v>900</v>
+      </c>
+      <c r="E62" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -1626,8 +2009,14 @@
       <c r="C63" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D63">
+        <v>80</v>
+      </c>
+      <c r="E63" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -1637,8 +2026,14 @@
       <c r="C64" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D64">
+        <v>80</v>
+      </c>
+      <c r="E64" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -1648,8 +2043,14 @@
       <c r="C65" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D65">
+        <v>80</v>
+      </c>
+      <c r="E65" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -1659,8 +2060,14 @@
       <c r="C66" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D66">
+        <v>120</v>
+      </c>
+      <c r="E66" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -1670,8 +2077,14 @@
       <c r="C67" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D67">
+        <v>120</v>
+      </c>
+      <c r="E67" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -1681,8 +2094,14 @@
       <c r="C68" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D68">
+        <v>120</v>
+      </c>
+      <c r="E68" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -1692,8 +2111,14 @@
       <c r="C69" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D69">
+        <v>80</v>
+      </c>
+      <c r="E69" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -1703,8 +2128,14 @@
       <c r="C70" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D70">
+        <v>80</v>
+      </c>
+      <c r="E70" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -1714,8 +2145,14 @@
       <c r="C71" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D71">
+        <v>80</v>
+      </c>
+      <c r="E71" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -1725,8 +2162,14 @@
       <c r="C72" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D72">
+        <v>80</v>
+      </c>
+      <c r="E72" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -1736,8 +2179,14 @@
       <c r="C73" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D73">
+        <v>80</v>
+      </c>
+      <c r="E73" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -1747,8 +2196,14 @@
       <c r="C74" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D74">
+        <v>80</v>
+      </c>
+      <c r="E74" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -1758,8 +2213,14 @@
       <c r="C75" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D75">
+        <v>80</v>
+      </c>
+      <c r="E75" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -1769,8 +2230,14 @@
       <c r="C76" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D76">
+        <v>80</v>
+      </c>
+      <c r="E76" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -1780,8 +2247,14 @@
       <c r="C77" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D77">
+        <v>120</v>
+      </c>
+      <c r="E77" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -1791,8 +2264,14 @@
       <c r="C78" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D78">
+        <v>450</v>
+      </c>
+      <c r="E78" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -1802,8 +2281,14 @@
       <c r="C79" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D79">
+        <v>450</v>
+      </c>
+      <c r="E79" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -1813,8 +2298,14 @@
       <c r="C80" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D80">
+        <v>450</v>
+      </c>
+      <c r="E80" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -1824,8 +2315,14 @@
       <c r="C81" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D81">
+        <v>450</v>
+      </c>
+      <c r="E81" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -1835,8 +2332,14 @@
       <c r="C82" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D82">
+        <v>450</v>
+      </c>
+      <c r="E82" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -1846,8 +2349,14 @@
       <c r="C83" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D83">
+        <v>450</v>
+      </c>
+      <c r="E83" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -1857,8 +2366,14 @@
       <c r="C84" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D84">
+        <v>450</v>
+      </c>
+      <c r="E84" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -1868,8 +2383,14 @@
       <c r="C85" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D85">
+        <v>450</v>
+      </c>
+      <c r="E85" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -1879,8 +2400,14 @@
       <c r="C86" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D86">
+        <v>450</v>
+      </c>
+      <c r="E86" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -1890,8 +2417,14 @@
       <c r="C87" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D87">
+        <v>450</v>
+      </c>
+      <c r="E87" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -1901,8 +2434,14 @@
       <c r="C88" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D88">
+        <v>450</v>
+      </c>
+      <c r="E88" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -1912,8 +2451,14 @@
       <c r="C89" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D89">
+        <v>120</v>
+      </c>
+      <c r="E89" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -1923,8 +2468,14 @@
       <c r="C90" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D90">
+        <v>900</v>
+      </c>
+      <c r="E90" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -1934,8 +2485,14 @@
       <c r="C91" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D91">
+        <v>900</v>
+      </c>
+      <c r="E91" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -1945,8 +2502,14 @@
       <c r="C92" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D92">
+        <v>900</v>
+      </c>
+      <c r="E92" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -1956,8 +2519,14 @@
       <c r="C93" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D93">
+        <v>80</v>
+      </c>
+      <c r="E93" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -1967,8 +2536,14 @@
       <c r="C94" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D94">
+        <v>900</v>
+      </c>
+      <c r="E94" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -1978,8 +2553,14 @@
       <c r="C95" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D95">
+        <v>80</v>
+      </c>
+      <c r="E95" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -1989,8 +2570,14 @@
       <c r="C96" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D96">
+        <v>120</v>
+      </c>
+      <c r="E96" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -2000,8 +2587,14 @@
       <c r="C97" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D97">
+        <v>450</v>
+      </c>
+      <c r="E97" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -2011,8 +2604,14 @@
       <c r="C98" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D98">
+        <v>450</v>
+      </c>
+      <c r="E98" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -2022,8 +2621,14 @@
       <c r="C99" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D99">
+        <v>450</v>
+      </c>
+      <c r="E99" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -2033,8 +2638,14 @@
       <c r="C100" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D100">
+        <v>450</v>
+      </c>
+      <c r="E100" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -2044,8 +2655,14 @@
       <c r="C101" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D101">
+        <v>450</v>
+      </c>
+      <c r="E101" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -2055,8 +2672,14 @@
       <c r="C102" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D102">
+        <v>450</v>
+      </c>
+      <c r="E102" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -2066,8 +2689,14 @@
       <c r="C103" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D103">
+        <v>450</v>
+      </c>
+      <c r="E103" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
@@ -2077,8 +2706,14 @@
       <c r="C104" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D104">
+        <v>450</v>
+      </c>
+      <c r="E104" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -2088,8 +2723,14 @@
       <c r="C105" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D105">
+        <v>120</v>
+      </c>
+      <c r="E105" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -2099,8 +2740,14 @@
       <c r="C106" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D106">
+        <v>80</v>
+      </c>
+      <c r="E106" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -2110,8 +2757,14 @@
       <c r="C107" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D107">
+        <v>80</v>
+      </c>
+      <c r="E107" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
@@ -2121,8 +2774,14 @@
       <c r="C108" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D108">
+        <v>80</v>
+      </c>
+      <c r="E108" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
@@ -2132,8 +2791,14 @@
       <c r="C109" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D109">
+        <v>80</v>
+      </c>
+      <c r="E109" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -2143,8 +2808,14 @@
       <c r="C110" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D110">
+        <v>80</v>
+      </c>
+      <c r="E110" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
@@ -2154,8 +2825,14 @@
       <c r="C111" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D111">
+        <v>80</v>
+      </c>
+      <c r="E111" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
@@ -2165,8 +2842,14 @@
       <c r="C112" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D112">
+        <v>80</v>
+      </c>
+      <c r="E112" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -2176,8 +2859,14 @@
       <c r="C113" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D113">
+        <v>80</v>
+      </c>
+      <c r="E113" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
@@ -2187,8 +2876,14 @@
       <c r="C114" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D114">
+        <v>900</v>
+      </c>
+      <c r="E114" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -2198,8 +2893,14 @@
       <c r="C115" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D115">
+        <v>450</v>
+      </c>
+      <c r="E115" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -2209,8 +2910,14 @@
       <c r="C116" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D116">
+        <v>450</v>
+      </c>
+      <c r="E116" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
@@ -2220,8 +2927,14 @@
       <c r="C117" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D117">
+        <v>450</v>
+      </c>
+      <c r="E117" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>117</v>
       </c>
@@ -2231,8 +2944,14 @@
       <c r="C118" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D118">
+        <v>450</v>
+      </c>
+      <c r="E118" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
@@ -2242,8 +2961,14 @@
       <c r="C119" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D119">
+        <v>450</v>
+      </c>
+      <c r="E119" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
@@ -2253,8 +2978,14 @@
       <c r="C120" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D120">
+        <v>450</v>
+      </c>
+      <c r="E120" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
@@ -2264,8 +2995,14 @@
       <c r="C121" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D121">
+        <v>450</v>
+      </c>
+      <c r="E121" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
@@ -2275,8 +3012,14 @@
       <c r="C122" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D122">
+        <v>450</v>
+      </c>
+      <c r="E122" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>122</v>
       </c>
@@ -2286,8 +3029,14 @@
       <c r="C123" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D123">
+        <v>450</v>
+      </c>
+      <c r="E123" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>123</v>
       </c>
@@ -2297,8 +3046,14 @@
       <c r="C124" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D124">
+        <v>450</v>
+      </c>
+      <c r="E124" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>124</v>
       </c>
@@ -2308,8 +3063,14 @@
       <c r="C125" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D125">
+        <v>450</v>
+      </c>
+      <c r="E125" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>125</v>
       </c>
@@ -2319,8 +3080,14 @@
       <c r="C126" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D126">
+        <v>120</v>
+      </c>
+      <c r="E126" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>126</v>
       </c>
@@ -2330,8 +3097,14 @@
       <c r="C127" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D127">
+        <v>900</v>
+      </c>
+      <c r="E127" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
       </c>
@@ -2341,8 +3114,14 @@
       <c r="C128" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D128">
+        <v>80</v>
+      </c>
+      <c r="E128" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>128</v>
       </c>
@@ -2352,8 +3131,14 @@
       <c r="C129" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D129">
+        <v>450</v>
+      </c>
+      <c r="E129" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>129</v>
       </c>
@@ -2363,8 +3148,14 @@
       <c r="C130" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D130">
+        <v>120</v>
+      </c>
+      <c r="E130" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>130</v>
       </c>
@@ -2374,8 +3165,14 @@
       <c r="C131" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D131">
+        <v>80</v>
+      </c>
+      <c r="E131" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>131</v>
       </c>
@@ -2385,8 +3182,14 @@
       <c r="C132" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D132">
+        <v>80</v>
+      </c>
+      <c r="E132" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>132</v>
       </c>
@@ -2396,8 +3199,14 @@
       <c r="C133" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D133">
+        <v>80</v>
+      </c>
+      <c r="E133" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>133</v>
       </c>
@@ -2407,8 +3216,14 @@
       <c r="C134" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D134">
+        <v>120</v>
+      </c>
+      <c r="E134" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>134</v>
       </c>
@@ -2418,8 +3233,14 @@
       <c r="C135" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D135">
+        <v>450</v>
+      </c>
+      <c r="E135" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>135</v>
       </c>
@@ -2429,8 +3250,14 @@
       <c r="C136" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D136">
+        <v>450</v>
+      </c>
+      <c r="E136" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>136</v>
       </c>
@@ -2440,8 +3267,14 @@
       <c r="C137" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D137">
+        <v>450</v>
+      </c>
+      <c r="E137" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>137</v>
       </c>
@@ -2451,8 +3284,14 @@
       <c r="C138" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D138">
+        <v>450</v>
+      </c>
+      <c r="E138" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>138</v>
       </c>
@@ -2462,8 +3301,14 @@
       <c r="C139" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D139">
+        <v>450</v>
+      </c>
+      <c r="E139" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>139</v>
       </c>
@@ -2473,8 +3318,14 @@
       <c r="C140" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D140">
+        <v>900</v>
+      </c>
+      <c r="E140" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>140</v>
       </c>
@@ -2484,8 +3335,14 @@
       <c r="C141" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D141">
+        <v>80</v>
+      </c>
+      <c r="E141" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>141</v>
       </c>
@@ -2495,8 +3352,14 @@
       <c r="C142" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D142">
+        <v>80</v>
+      </c>
+      <c r="E142" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>142</v>
       </c>
@@ -2506,8 +3369,14 @@
       <c r="C143" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D143">
+        <v>80</v>
+      </c>
+      <c r="E143" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>143</v>
       </c>
@@ -2517,8 +3386,14 @@
       <c r="C144" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D144">
+        <v>900</v>
+      </c>
+      <c r="E144" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>144</v>
       </c>
@@ -2528,8 +3403,14 @@
       <c r="C145" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D145">
+        <v>120</v>
+      </c>
+      <c r="E145" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>145</v>
       </c>
@@ -2539,8 +3420,14 @@
       <c r="C146" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D146">
+        <v>80</v>
+      </c>
+      <c r="E146" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>146</v>
       </c>
@@ -2550,8 +3437,14 @@
       <c r="C147" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D147">
+        <v>900</v>
+      </c>
+      <c r="E147" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>147</v>
       </c>
@@ -2561,8 +3454,14 @@
       <c r="C148" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D148">
+        <v>450</v>
+      </c>
+      <c r="E148" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>148</v>
       </c>
@@ -2572,8 +3471,14 @@
       <c r="C149" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D149">
+        <v>80</v>
+      </c>
+      <c r="E149" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>149</v>
       </c>
@@ -2583,8 +3488,14 @@
       <c r="C150" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D150">
+        <v>80</v>
+      </c>
+      <c r="E150" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>150</v>
       </c>
@@ -2594,8 +3505,14 @@
       <c r="C151" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D151">
+        <v>80</v>
+      </c>
+      <c r="E151" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>151</v>
       </c>
@@ -2605,8 +3522,14 @@
       <c r="C152" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D152">
+        <v>80</v>
+      </c>
+      <c r="E152" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>152</v>
       </c>
@@ -2615,6 +3538,21 @@
       </c>
       <c r="C153" t="s">
         <v>167</v>
+      </c>
+      <c r="D153">
+        <v>900</v>
+      </c>
+      <c r="E153" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D154">
+        <f>SUM(D2:D153)</f>
+        <v>55930</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
base de dados alteraçao no mes da aplicação
</commit_message>
<xml_diff>
--- a/base de dados.xlsx
+++ b/base de dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesle\Desktop\Projeto-Power-BI-Oficina-Mecanica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{185D673A-788A-408E-8B03-85C8EB602BBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17B75B1D-BFC6-4E89-9C37-D526395A817D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11640" xr2:uid="{C68C1244-3D4F-43FC-8114-B501E2A75E8B}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="178">
   <si>
     <t>ID_Cliente</t>
   </si>
@@ -560,16 +560,40 @@
   </si>
   <si>
     <t>Serviço</t>
+  </si>
+  <si>
+    <t>Mês</t>
+  </si>
+  <si>
+    <t>Janeiro</t>
+  </si>
+  <si>
+    <t>Fevereiro</t>
+  </si>
+  <si>
+    <t>Março</t>
+  </si>
+  <si>
+    <t>Abril</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -595,10 +619,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -935,17 +962,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47DEE4CA-CEFF-4D30-B427-5B29E0AA61DD}">
-  <dimension ref="A1:E154"/>
+  <dimension ref="A1:F154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -955,14 +983,17 @@
       <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>171</v>
       </c>
       <c r="E1" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -972,14 +1003,17 @@
       <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="3">
         <v>900</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -989,14 +1023,17 @@
       <c r="C3" t="s">
         <v>167</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="3">
         <v>120</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1006,14 +1043,17 @@
       <c r="C4" t="s">
         <v>168</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="3">
         <v>120</v>
       </c>
       <c r="E4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1023,14 +1063,17 @@
       <c r="C5" t="s">
         <v>169</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="3">
         <v>900</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1040,14 +1083,17 @@
       <c r="C6" t="s">
         <v>170</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="3">
         <v>900</v>
       </c>
       <c r="E6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1057,14 +1103,17 @@
       <c r="C7" t="s">
         <v>2</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="3">
         <v>80</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1074,14 +1123,17 @@
       <c r="C8" t="s">
         <v>167</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="3">
         <v>900</v>
       </c>
       <c r="E8" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1091,14 +1143,17 @@
       <c r="C9" t="s">
         <v>168</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="3">
         <v>120</v>
       </c>
       <c r="E9" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1108,14 +1163,17 @@
       <c r="C10" t="s">
         <v>169</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="3">
         <v>900</v>
       </c>
       <c r="E10" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1125,14 +1183,17 @@
       <c r="C11" t="s">
         <v>170</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="3">
         <v>900</v>
       </c>
       <c r="E11" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1142,14 +1203,17 @@
       <c r="C12" t="s">
         <v>2</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="3">
         <v>80</v>
       </c>
       <c r="E12" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1159,14 +1223,17 @@
       <c r="C13" t="s">
         <v>167</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="3">
         <v>80</v>
       </c>
       <c r="E13" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1176,14 +1243,17 @@
       <c r="C14" t="s">
         <v>168</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="3">
         <v>900</v>
       </c>
       <c r="E14" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1193,14 +1263,17 @@
       <c r="C15" t="s">
         <v>169</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="3">
         <v>80</v>
       </c>
       <c r="E15" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1210,14 +1283,17 @@
       <c r="C16" t="s">
         <v>170</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="3">
         <v>900</v>
       </c>
       <c r="E16" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1227,14 +1303,17 @@
       <c r="C17" t="s">
         <v>2</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="3">
         <v>80</v>
       </c>
       <c r="E17" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1244,14 +1323,17 @@
       <c r="C18" t="s">
         <v>167</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="3">
         <v>80</v>
       </c>
       <c r="E18" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1261,14 +1343,17 @@
       <c r="C19" t="s">
         <v>168</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="3">
         <v>900</v>
       </c>
       <c r="E19" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1278,14 +1363,17 @@
       <c r="C20" t="s">
         <v>169</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="3">
         <v>80</v>
       </c>
       <c r="E20" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1295,14 +1383,17 @@
       <c r="C21" t="s">
         <v>170</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="3">
         <v>80</v>
       </c>
       <c r="E21" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1312,14 +1403,17 @@
       <c r="C22" t="s">
         <v>2</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="3">
         <v>900</v>
       </c>
       <c r="E22" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1329,14 +1423,17 @@
       <c r="C23" t="s">
         <v>167</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="3">
         <v>900</v>
       </c>
       <c r="E23" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1346,14 +1443,17 @@
       <c r="C24" t="s">
         <v>168</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="3">
         <v>120</v>
       </c>
       <c r="E24" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1363,14 +1463,17 @@
       <c r="C25" t="s">
         <v>169</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="3">
         <v>120</v>
       </c>
       <c r="E25" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1380,14 +1483,17 @@
       <c r="C26" t="s">
         <v>170</v>
       </c>
-      <c r="D26">
+      <c r="D26" s="3">
         <v>120</v>
       </c>
       <c r="E26" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1397,14 +1503,17 @@
       <c r="C27" t="s">
         <v>2</v>
       </c>
-      <c r="D27">
+      <c r="D27" s="3">
         <v>120</v>
       </c>
       <c r="E27" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1414,14 +1523,17 @@
       <c r="C28" t="s">
         <v>167</v>
       </c>
-      <c r="D28">
+      <c r="D28" s="3">
         <v>120</v>
       </c>
       <c r="E28" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1431,14 +1543,17 @@
       <c r="C29" t="s">
         <v>168</v>
       </c>
-      <c r="D29">
+      <c r="D29" s="3">
         <v>900</v>
       </c>
       <c r="E29" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1448,14 +1563,17 @@
       <c r="C30" t="s">
         <v>169</v>
       </c>
-      <c r="D30">
+      <c r="D30" s="3">
         <v>300</v>
       </c>
       <c r="E30" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1465,14 +1583,17 @@
       <c r="C31" t="s">
         <v>170</v>
       </c>
-      <c r="D31">
+      <c r="D31" s="3">
         <v>300</v>
       </c>
       <c r="E31" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1482,14 +1603,17 @@
       <c r="C32" t="s">
         <v>2</v>
       </c>
-      <c r="D32">
+      <c r="D32" s="3">
         <v>300</v>
       </c>
       <c r="E32" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1499,14 +1623,17 @@
       <c r="C33" t="s">
         <v>167</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="3">
         <v>300</v>
       </c>
       <c r="E33" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1516,14 +1643,17 @@
       <c r="C34" t="s">
         <v>168</v>
       </c>
-      <c r="D34">
+      <c r="D34" s="3">
         <v>300</v>
       </c>
       <c r="E34" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1533,14 +1663,17 @@
       <c r="C35" t="s">
         <v>169</v>
       </c>
-      <c r="D35">
+      <c r="D35" s="3">
         <v>900</v>
       </c>
       <c r="E35" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1550,14 +1683,17 @@
       <c r="C36" t="s">
         <v>170</v>
       </c>
-      <c r="D36">
+      <c r="D36" s="3">
         <v>450</v>
       </c>
       <c r="E36" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1567,14 +1703,17 @@
       <c r="C37" t="s">
         <v>2</v>
       </c>
-      <c r="D37">
+      <c r="D37" s="3">
         <v>450</v>
       </c>
       <c r="E37" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1584,14 +1723,17 @@
       <c r="C38" t="s">
         <v>167</v>
       </c>
-      <c r="D38">
+      <c r="D38" s="3">
         <v>450</v>
       </c>
       <c r="E38" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1601,14 +1743,17 @@
       <c r="C39" t="s">
         <v>168</v>
       </c>
-      <c r="D39">
+      <c r="D39" s="3">
         <v>900</v>
       </c>
       <c r="E39" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1618,14 +1763,17 @@
       <c r="C40" t="s">
         <v>169</v>
       </c>
-      <c r="D40">
+      <c r="D40" s="3">
         <v>450</v>
       </c>
       <c r="E40" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1635,14 +1783,17 @@
       <c r="C41" t="s">
         <v>170</v>
       </c>
-      <c r="D41">
+      <c r="D41" s="3">
         <v>450</v>
       </c>
       <c r="E41" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1652,14 +1803,17 @@
       <c r="C42" t="s">
         <v>2</v>
       </c>
-      <c r="D42">
+      <c r="D42" s="3">
         <v>450</v>
       </c>
       <c r="E42" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1669,14 +1823,17 @@
       <c r="C43" t="s">
         <v>167</v>
       </c>
-      <c r="D43">
+      <c r="D43" s="3">
         <v>120</v>
       </c>
       <c r="E43" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1686,14 +1843,17 @@
       <c r="C44" t="s">
         <v>168</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="3">
         <v>120</v>
       </c>
       <c r="E44" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1703,14 +1863,17 @@
       <c r="C45" t="s">
         <v>169</v>
       </c>
-      <c r="D45">
+      <c r="D45" s="3">
         <v>120</v>
       </c>
       <c r="E45" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1720,14 +1883,17 @@
       <c r="C46" t="s">
         <v>170</v>
       </c>
-      <c r="D46">
+      <c r="D46" s="3">
         <v>120</v>
       </c>
       <c r="E46" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F46" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1737,14 +1903,17 @@
       <c r="C47" t="s">
         <v>2</v>
       </c>
-      <c r="D47">
+      <c r="D47" s="3">
         <v>120</v>
       </c>
       <c r="E47" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1754,14 +1923,17 @@
       <c r="C48" t="s">
         <v>167</v>
       </c>
-      <c r="D48">
+      <c r="D48" s="3">
         <v>120</v>
       </c>
       <c r="E48" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F48" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1771,14 +1943,17 @@
       <c r="C49" t="s">
         <v>168</v>
       </c>
-      <c r="D49">
+      <c r="D49" s="3">
         <v>450</v>
       </c>
       <c r="E49" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1788,14 +1963,17 @@
       <c r="C50" t="s">
         <v>169</v>
       </c>
-      <c r="D50">
+      <c r="D50" s="3">
         <v>450</v>
       </c>
       <c r="E50" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F50" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1805,14 +1983,17 @@
       <c r="C51" t="s">
         <v>170</v>
       </c>
-      <c r="D51">
+      <c r="D51" s="3">
         <v>450</v>
       </c>
       <c r="E51" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F51" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1822,14 +2003,17 @@
       <c r="C52" t="s">
         <v>2</v>
       </c>
-      <c r="D52">
+      <c r="D52" s="3">
         <v>450</v>
       </c>
       <c r="E52" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F52" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1839,14 +2023,17 @@
       <c r="C53" t="s">
         <v>167</v>
       </c>
-      <c r="D53">
+      <c r="D53" s="3">
         <v>900</v>
       </c>
       <c r="E53" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F53" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1856,14 +2043,17 @@
       <c r="C54" t="s">
         <v>168</v>
       </c>
-      <c r="D54">
+      <c r="D54" s="3">
         <v>450</v>
       </c>
       <c r="E54" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F54" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1873,14 +2063,17 @@
       <c r="C55" t="s">
         <v>169</v>
       </c>
-      <c r="D55">
+      <c r="D55" s="3">
         <v>450</v>
       </c>
       <c r="E55" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F55" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1890,14 +2083,17 @@
       <c r="C56" t="s">
         <v>170</v>
       </c>
-      <c r="D56">
+      <c r="D56" s="3">
         <v>450</v>
       </c>
       <c r="E56" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F56" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1907,14 +2103,17 @@
       <c r="C57" t="s">
         <v>2</v>
       </c>
-      <c r="D57">
+      <c r="D57" s="3">
         <v>450</v>
       </c>
       <c r="E57" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F57" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1924,14 +2123,17 @@
       <c r="C58" t="s">
         <v>167</v>
       </c>
-      <c r="D58">
+      <c r="D58" s="3">
         <v>450</v>
       </c>
       <c r="E58" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F58" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -1941,14 +2143,17 @@
       <c r="C59" t="s">
         <v>168</v>
       </c>
-      <c r="D59">
+      <c r="D59" s="3">
         <v>450</v>
       </c>
       <c r="E59" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F59" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -1958,14 +2163,17 @@
       <c r="C60" t="s">
         <v>169</v>
       </c>
-      <c r="D60">
+      <c r="D60" s="3">
         <v>450</v>
       </c>
       <c r="E60" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F60" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -1975,14 +2183,17 @@
       <c r="C61" t="s">
         <v>170</v>
       </c>
-      <c r="D61">
+      <c r="D61" s="3">
         <v>450</v>
       </c>
       <c r="E61" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F61" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -1992,14 +2203,17 @@
       <c r="C62" t="s">
         <v>2</v>
       </c>
-      <c r="D62">
+      <c r="D62" s="3">
         <v>900</v>
       </c>
       <c r="E62" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F62" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2009,14 +2223,17 @@
       <c r="C63" t="s">
         <v>167</v>
       </c>
-      <c r="D63">
+      <c r="D63" s="3">
         <v>80</v>
       </c>
       <c r="E63" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F63" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2026,14 +2243,17 @@
       <c r="C64" t="s">
         <v>168</v>
       </c>
-      <c r="D64">
+      <c r="D64" s="3">
         <v>80</v>
       </c>
       <c r="E64" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F64" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2043,14 +2263,17 @@
       <c r="C65" t="s">
         <v>169</v>
       </c>
-      <c r="D65">
+      <c r="D65" s="3">
         <v>80</v>
       </c>
       <c r="E65" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F65" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2060,14 +2283,17 @@
       <c r="C66" t="s">
         <v>170</v>
       </c>
-      <c r="D66">
+      <c r="D66" s="3">
         <v>120</v>
       </c>
       <c r="E66" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F66" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2077,14 +2303,17 @@
       <c r="C67" t="s">
         <v>2</v>
       </c>
-      <c r="D67">
+      <c r="D67" s="3">
         <v>120</v>
       </c>
       <c r="E67" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F67" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2094,14 +2323,17 @@
       <c r="C68" t="s">
         <v>167</v>
       </c>
-      <c r="D68">
+      <c r="D68" s="3">
         <v>120</v>
       </c>
       <c r="E68" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F68" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2111,14 +2343,17 @@
       <c r="C69" t="s">
         <v>168</v>
       </c>
-      <c r="D69">
+      <c r="D69" s="3">
         <v>80</v>
       </c>
       <c r="E69" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F69" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2128,14 +2363,17 @@
       <c r="C70" t="s">
         <v>169</v>
       </c>
-      <c r="D70">
+      <c r="D70" s="3">
         <v>80</v>
       </c>
       <c r="E70" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F70" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2145,14 +2383,17 @@
       <c r="C71" t="s">
         <v>170</v>
       </c>
-      <c r="D71">
+      <c r="D71" s="3">
         <v>80</v>
       </c>
       <c r="E71" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F71" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2162,14 +2403,17 @@
       <c r="C72" t="s">
         <v>2</v>
       </c>
-      <c r="D72">
+      <c r="D72" s="3">
         <v>80</v>
       </c>
       <c r="E72" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F72" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2179,14 +2423,17 @@
       <c r="C73" t="s">
         <v>167</v>
       </c>
-      <c r="D73">
+      <c r="D73" s="3">
         <v>80</v>
       </c>
       <c r="E73" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F73" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2196,14 +2443,17 @@
       <c r="C74" t="s">
         <v>168</v>
       </c>
-      <c r="D74">
+      <c r="D74" s="3">
         <v>80</v>
       </c>
       <c r="E74" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F74" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2213,14 +2463,17 @@
       <c r="C75" t="s">
         <v>169</v>
       </c>
-      <c r="D75">
+      <c r="D75" s="3">
         <v>80</v>
       </c>
       <c r="E75" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F75" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2230,14 +2483,17 @@
       <c r="C76" t="s">
         <v>170</v>
       </c>
-      <c r="D76">
+      <c r="D76" s="3">
         <v>80</v>
       </c>
       <c r="E76" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F76" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2247,14 +2503,17 @@
       <c r="C77" t="s">
         <v>2</v>
       </c>
-      <c r="D77">
+      <c r="D77" s="3">
         <v>120</v>
       </c>
       <c r="E77" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F77" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2264,14 +2523,17 @@
       <c r="C78" t="s">
         <v>167</v>
       </c>
-      <c r="D78">
+      <c r="D78" s="3">
         <v>450</v>
       </c>
       <c r="E78" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F78" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2281,14 +2543,17 @@
       <c r="C79" t="s">
         <v>168</v>
       </c>
-      <c r="D79">
+      <c r="D79" s="3">
         <v>450</v>
       </c>
       <c r="E79" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F79" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2298,14 +2563,17 @@
       <c r="C80" t="s">
         <v>169</v>
       </c>
-      <c r="D80">
+      <c r="D80" s="3">
         <v>450</v>
       </c>
       <c r="E80" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F80" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2315,14 +2583,17 @@
       <c r="C81" t="s">
         <v>170</v>
       </c>
-      <c r="D81">
+      <c r="D81" s="3">
         <v>450</v>
       </c>
       <c r="E81" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F81" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2332,14 +2603,17 @@
       <c r="C82" t="s">
         <v>2</v>
       </c>
-      <c r="D82">
+      <c r="D82" s="3">
         <v>450</v>
       </c>
       <c r="E82" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F82" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2349,14 +2623,17 @@
       <c r="C83" t="s">
         <v>167</v>
       </c>
-      <c r="D83">
+      <c r="D83" s="3">
         <v>450</v>
       </c>
       <c r="E83" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F83" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2366,14 +2643,17 @@
       <c r="C84" t="s">
         <v>168</v>
       </c>
-      <c r="D84">
+      <c r="D84" s="3">
         <v>450</v>
       </c>
       <c r="E84" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F84" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2383,14 +2663,17 @@
       <c r="C85" t="s">
         <v>169</v>
       </c>
-      <c r="D85">
+      <c r="D85" s="3">
         <v>450</v>
       </c>
       <c r="E85" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F85" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2400,14 +2683,17 @@
       <c r="C86" t="s">
         <v>170</v>
       </c>
-      <c r="D86">
+      <c r="D86" s="3">
         <v>450</v>
       </c>
       <c r="E86" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F86" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2417,14 +2703,17 @@
       <c r="C87" t="s">
         <v>2</v>
       </c>
-      <c r="D87">
+      <c r="D87" s="3">
         <v>450</v>
       </c>
       <c r="E87" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F87" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2434,14 +2723,17 @@
       <c r="C88" t="s">
         <v>167</v>
       </c>
-      <c r="D88">
+      <c r="D88" s="3">
         <v>450</v>
       </c>
       <c r="E88" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F88" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2451,14 +2743,17 @@
       <c r="C89" t="s">
         <v>168</v>
       </c>
-      <c r="D89">
+      <c r="D89" s="3">
         <v>120</v>
       </c>
       <c r="E89" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F89" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2468,14 +2763,17 @@
       <c r="C90" t="s">
         <v>169</v>
       </c>
-      <c r="D90">
+      <c r="D90" s="3">
         <v>900</v>
       </c>
       <c r="E90" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F90" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2485,14 +2783,17 @@
       <c r="C91" t="s">
         <v>170</v>
       </c>
-      <c r="D91">
+      <c r="D91" s="3">
         <v>900</v>
       </c>
       <c r="E91" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F91" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2502,14 +2803,17 @@
       <c r="C92" t="s">
         <v>2</v>
       </c>
-      <c r="D92">
+      <c r="D92" s="3">
         <v>900</v>
       </c>
       <c r="E92" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F92" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2519,14 +2823,17 @@
       <c r="C93" t="s">
         <v>167</v>
       </c>
-      <c r="D93">
+      <c r="D93" s="3">
         <v>80</v>
       </c>
       <c r="E93" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F93" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2536,14 +2843,17 @@
       <c r="C94" t="s">
         <v>168</v>
       </c>
-      <c r="D94">
+      <c r="D94" s="3">
         <v>900</v>
       </c>
       <c r="E94" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F94" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -2553,14 +2863,17 @@
       <c r="C95" t="s">
         <v>169</v>
       </c>
-      <c r="D95">
+      <c r="D95" s="3">
         <v>80</v>
       </c>
       <c r="E95" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F95" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -2570,14 +2883,17 @@
       <c r="C96" t="s">
         <v>170</v>
       </c>
-      <c r="D96">
+      <c r="D96" s="3">
         <v>120</v>
       </c>
       <c r="E96" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F96" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -2587,14 +2903,17 @@
       <c r="C97" t="s">
         <v>2</v>
       </c>
-      <c r="D97">
+      <c r="D97" s="3">
         <v>450</v>
       </c>
       <c r="E97" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F97" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -2604,14 +2923,17 @@
       <c r="C98" t="s">
         <v>167</v>
       </c>
-      <c r="D98">
+      <c r="D98" s="3">
         <v>450</v>
       </c>
       <c r="E98" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F98" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -2621,14 +2943,17 @@
       <c r="C99" t="s">
         <v>168</v>
       </c>
-      <c r="D99">
+      <c r="D99" s="3">
         <v>450</v>
       </c>
       <c r="E99" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F99" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -2638,14 +2963,17 @@
       <c r="C100" t="s">
         <v>169</v>
       </c>
-      <c r="D100">
+      <c r="D100" s="3">
         <v>450</v>
       </c>
       <c r="E100" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F100" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -2655,14 +2983,17 @@
       <c r="C101" t="s">
         <v>170</v>
       </c>
-      <c r="D101">
+      <c r="D101" s="3">
         <v>450</v>
       </c>
       <c r="E101" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F101" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -2672,14 +3003,17 @@
       <c r="C102" t="s">
         <v>2</v>
       </c>
-      <c r="D102">
+      <c r="D102" s="3">
         <v>450</v>
       </c>
       <c r="E102" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F102" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -2689,14 +3023,17 @@
       <c r="C103" t="s">
         <v>167</v>
       </c>
-      <c r="D103">
+      <c r="D103" s="3">
         <v>450</v>
       </c>
       <c r="E103" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F103" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
@@ -2706,14 +3043,17 @@
       <c r="C104" t="s">
         <v>168</v>
       </c>
-      <c r="D104">
+      <c r="D104" s="3">
         <v>450</v>
       </c>
       <c r="E104" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F104" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -2723,14 +3063,17 @@
       <c r="C105" t="s">
         <v>169</v>
       </c>
-      <c r="D105">
+      <c r="D105" s="3">
         <v>120</v>
       </c>
       <c r="E105" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F105" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -2740,14 +3083,17 @@
       <c r="C106" t="s">
         <v>170</v>
       </c>
-      <c r="D106">
+      <c r="D106" s="3">
         <v>80</v>
       </c>
       <c r="E106" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F106" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -2757,14 +3103,17 @@
       <c r="C107" t="s">
         <v>2</v>
       </c>
-      <c r="D107">
+      <c r="D107" s="3">
         <v>80</v>
       </c>
       <c r="E107" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F107" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
@@ -2774,14 +3123,17 @@
       <c r="C108" t="s">
         <v>167</v>
       </c>
-      <c r="D108">
+      <c r="D108" s="3">
         <v>80</v>
       </c>
       <c r="E108" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F108" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
@@ -2791,14 +3143,17 @@
       <c r="C109" t="s">
         <v>168</v>
       </c>
-      <c r="D109">
+      <c r="D109" s="3">
         <v>80</v>
       </c>
       <c r="E109" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F109" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -2808,14 +3163,17 @@
       <c r="C110" t="s">
         <v>169</v>
       </c>
-      <c r="D110">
+      <c r="D110" s="3">
         <v>80</v>
       </c>
       <c r="E110" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F110" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
@@ -2825,14 +3183,17 @@
       <c r="C111" t="s">
         <v>170</v>
       </c>
-      <c r="D111">
+      <c r="D111" s="3">
         <v>80</v>
       </c>
       <c r="E111" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F111" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
@@ -2842,14 +3203,17 @@
       <c r="C112" t="s">
         <v>2</v>
       </c>
-      <c r="D112">
+      <c r="D112" s="3">
         <v>80</v>
       </c>
       <c r="E112" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F112" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -2859,14 +3223,17 @@
       <c r="C113" t="s">
         <v>167</v>
       </c>
-      <c r="D113">
+      <c r="D113" s="3">
         <v>80</v>
       </c>
       <c r="E113" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F113" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
@@ -2876,14 +3243,17 @@
       <c r="C114" t="s">
         <v>168</v>
       </c>
-      <c r="D114">
+      <c r="D114" s="3">
         <v>900</v>
       </c>
       <c r="E114" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F114" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -2893,14 +3263,17 @@
       <c r="C115" t="s">
         <v>169</v>
       </c>
-      <c r="D115">
+      <c r="D115" s="3">
         <v>450</v>
       </c>
       <c r="E115" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F115" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -2910,14 +3283,17 @@
       <c r="C116" t="s">
         <v>170</v>
       </c>
-      <c r="D116">
+      <c r="D116" s="3">
         <v>450</v>
       </c>
       <c r="E116" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F116" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
@@ -2927,14 +3303,17 @@
       <c r="C117" t="s">
         <v>2</v>
       </c>
-      <c r="D117">
+      <c r="D117" s="3">
         <v>450</v>
       </c>
       <c r="E117" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F117" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>117</v>
       </c>
@@ -2944,14 +3323,17 @@
       <c r="C118" t="s">
         <v>167</v>
       </c>
-      <c r="D118">
+      <c r="D118" s="3">
         <v>450</v>
       </c>
       <c r="E118" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F118" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
@@ -2961,14 +3343,17 @@
       <c r="C119" t="s">
         <v>168</v>
       </c>
-      <c r="D119">
+      <c r="D119" s="3">
         <v>450</v>
       </c>
       <c r="E119" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F119" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
@@ -2978,14 +3363,17 @@
       <c r="C120" t="s">
         <v>169</v>
       </c>
-      <c r="D120">
+      <c r="D120" s="3">
         <v>450</v>
       </c>
       <c r="E120" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F120" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
@@ -2995,14 +3383,17 @@
       <c r="C121" t="s">
         <v>170</v>
       </c>
-      <c r="D121">
+      <c r="D121" s="3">
         <v>450</v>
       </c>
       <c r="E121" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F121" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
@@ -3012,14 +3403,17 @@
       <c r="C122" t="s">
         <v>2</v>
       </c>
-      <c r="D122">
+      <c r="D122" s="3">
         <v>450</v>
       </c>
       <c r="E122" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F122" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>122</v>
       </c>
@@ -3029,14 +3423,17 @@
       <c r="C123" t="s">
         <v>167</v>
       </c>
-      <c r="D123">
+      <c r="D123" s="3">
         <v>450</v>
       </c>
       <c r="E123" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F123" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>123</v>
       </c>
@@ -3046,14 +3443,17 @@
       <c r="C124" t="s">
         <v>168</v>
       </c>
-      <c r="D124">
+      <c r="D124" s="3">
         <v>450</v>
       </c>
       <c r="E124" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F124" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>124</v>
       </c>
@@ -3063,14 +3463,17 @@
       <c r="C125" t="s">
         <v>169</v>
       </c>
-      <c r="D125">
+      <c r="D125" s="3">
         <v>450</v>
       </c>
       <c r="E125" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F125" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>125</v>
       </c>
@@ -3080,14 +3483,17 @@
       <c r="C126" t="s">
         <v>170</v>
       </c>
-      <c r="D126">
+      <c r="D126" s="3">
         <v>120</v>
       </c>
       <c r="E126" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F126" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>126</v>
       </c>
@@ -3097,14 +3503,17 @@
       <c r="C127" t="s">
         <v>2</v>
       </c>
-      <c r="D127">
+      <c r="D127" s="3">
         <v>900</v>
       </c>
       <c r="E127" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F127" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
       </c>
@@ -3114,14 +3523,17 @@
       <c r="C128" t="s">
         <v>167</v>
       </c>
-      <c r="D128">
+      <c r="D128" s="3">
         <v>80</v>
       </c>
       <c r="E128" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F128" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>128</v>
       </c>
@@ -3131,14 +3543,17 @@
       <c r="C129" t="s">
         <v>168</v>
       </c>
-      <c r="D129">
+      <c r="D129" s="3">
         <v>450</v>
       </c>
       <c r="E129" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F129" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>129</v>
       </c>
@@ -3148,14 +3563,17 @@
       <c r="C130" t="s">
         <v>169</v>
       </c>
-      <c r="D130">
+      <c r="D130" s="3">
         <v>120</v>
       </c>
       <c r="E130" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F130" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>130</v>
       </c>
@@ -3165,14 +3583,17 @@
       <c r="C131" t="s">
         <v>170</v>
       </c>
-      <c r="D131">
+      <c r="D131" s="3">
         <v>80</v>
       </c>
       <c r="E131" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F131" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>131</v>
       </c>
@@ -3182,14 +3603,17 @@
       <c r="C132" t="s">
         <v>2</v>
       </c>
-      <c r="D132">
+      <c r="D132" s="3">
         <v>80</v>
       </c>
       <c r="E132" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F132" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>132</v>
       </c>
@@ -3199,14 +3623,17 @@
       <c r="C133" t="s">
         <v>167</v>
       </c>
-      <c r="D133">
+      <c r="D133" s="3">
         <v>80</v>
       </c>
       <c r="E133" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F133" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>133</v>
       </c>
@@ -3216,14 +3643,17 @@
       <c r="C134" t="s">
         <v>168</v>
       </c>
-      <c r="D134">
+      <c r="D134" s="3">
         <v>120</v>
       </c>
       <c r="E134" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F134" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>134</v>
       </c>
@@ -3233,14 +3663,17 @@
       <c r="C135" t="s">
         <v>169</v>
       </c>
-      <c r="D135">
+      <c r="D135" s="3">
         <v>450</v>
       </c>
       <c r="E135" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F135" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>135</v>
       </c>
@@ -3250,14 +3683,17 @@
       <c r="C136" t="s">
         <v>170</v>
       </c>
-      <c r="D136">
+      <c r="D136" s="3">
         <v>450</v>
       </c>
       <c r="E136" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F136" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>136</v>
       </c>
@@ -3267,14 +3703,17 @@
       <c r="C137" t="s">
         <v>2</v>
       </c>
-      <c r="D137">
+      <c r="D137" s="3">
         <v>450</v>
       </c>
       <c r="E137" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F137" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>137</v>
       </c>
@@ -3284,14 +3723,17 @@
       <c r="C138" t="s">
         <v>167</v>
       </c>
-      <c r="D138">
+      <c r="D138" s="3">
         <v>450</v>
       </c>
       <c r="E138" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F138" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>138</v>
       </c>
@@ -3301,14 +3743,17 @@
       <c r="C139" t="s">
         <v>168</v>
       </c>
-      <c r="D139">
+      <c r="D139" s="3">
         <v>450</v>
       </c>
       <c r="E139" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F139" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>139</v>
       </c>
@@ -3318,14 +3763,17 @@
       <c r="C140" t="s">
         <v>169</v>
       </c>
-      <c r="D140">
+      <c r="D140" s="3">
         <v>900</v>
       </c>
       <c r="E140" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F140" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>140</v>
       </c>
@@ -3335,14 +3783,17 @@
       <c r="C141" t="s">
         <v>170</v>
       </c>
-      <c r="D141">
+      <c r="D141" s="3">
         <v>80</v>
       </c>
       <c r="E141" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F141" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>141</v>
       </c>
@@ -3352,14 +3803,17 @@
       <c r="C142" t="s">
         <v>2</v>
       </c>
-      <c r="D142">
+      <c r="D142" s="3">
         <v>80</v>
       </c>
       <c r="E142" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F142" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>142</v>
       </c>
@@ -3369,14 +3823,17 @@
       <c r="C143" t="s">
         <v>167</v>
       </c>
-      <c r="D143">
+      <c r="D143" s="3">
         <v>80</v>
       </c>
       <c r="E143" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F143" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>143</v>
       </c>
@@ -3386,14 +3843,17 @@
       <c r="C144" t="s">
         <v>168</v>
       </c>
-      <c r="D144">
+      <c r="D144" s="3">
         <v>900</v>
       </c>
       <c r="E144" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F144" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>144</v>
       </c>
@@ -3403,14 +3863,17 @@
       <c r="C145" t="s">
         <v>169</v>
       </c>
-      <c r="D145">
+      <c r="D145" s="3">
         <v>120</v>
       </c>
       <c r="E145" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F145" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>145</v>
       </c>
@@ -3420,14 +3883,17 @@
       <c r="C146" t="s">
         <v>170</v>
       </c>
-      <c r="D146">
+      <c r="D146" s="3">
         <v>80</v>
       </c>
       <c r="E146" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F146" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>146</v>
       </c>
@@ -3437,14 +3903,17 @@
       <c r="C147" t="s">
         <v>2</v>
       </c>
-      <c r="D147">
+      <c r="D147" s="3">
         <v>900</v>
       </c>
       <c r="E147" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F147" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>147</v>
       </c>
@@ -3454,14 +3923,17 @@
       <c r="C148" t="s">
         <v>167</v>
       </c>
-      <c r="D148">
+      <c r="D148" s="3">
         <v>450</v>
       </c>
       <c r="E148" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F148" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>148</v>
       </c>
@@ -3471,14 +3943,17 @@
       <c r="C149" t="s">
         <v>168</v>
       </c>
-      <c r="D149">
+      <c r="D149" s="3">
         <v>80</v>
       </c>
       <c r="E149" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F149" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>149</v>
       </c>
@@ -3488,14 +3963,17 @@
       <c r="C150" t="s">
         <v>169</v>
       </c>
-      <c r="D150">
+      <c r="D150" s="3">
         <v>80</v>
       </c>
       <c r="E150" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F150" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>150</v>
       </c>
@@ -3505,14 +3983,17 @@
       <c r="C151" t="s">
         <v>170</v>
       </c>
-      <c r="D151">
+      <c r="D151" s="3">
         <v>80</v>
       </c>
       <c r="E151" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F151" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>151</v>
       </c>
@@ -3522,14 +4003,17 @@
       <c r="C152" t="s">
         <v>2</v>
       </c>
-      <c r="D152">
+      <c r="D152" s="3">
         <v>80</v>
       </c>
       <c r="E152" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F152" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>152</v>
       </c>
@@ -3539,23 +4023,27 @@
       <c r="C153" t="s">
         <v>167</v>
       </c>
-      <c r="D153">
+      <c r="D153" s="3">
         <v>900</v>
       </c>
       <c r="E153" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F153" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D154">
+      <c r="D154" s="3">
         <f>SUM(D2:D153)</f>
         <v>55930</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
delete base de dados
</commit_message>
<xml_diff>
--- a/base de dados.xlsx
+++ b/base de dados.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesle\Desktop\Projeto-Power-BI-Oficina-Mecanica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17B75B1D-BFC6-4E89-9C37-D526395A817D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4170130-4B6E-40EE-8B62-A71A9475B1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11640" xr2:uid="{C68C1244-3D4F-43FC-8114-B501E2A75E8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Cliente" sheetId="1" r:id="rId1"/>
     <sheet name="Serviços" sheetId="2" r:id="rId2"/>
-    <sheet name="Ordens de Serviço" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="174">
   <si>
     <t>ID_Cliente</t>
   </si>
@@ -79,19 +78,7 @@
     <t>Revisao geral</t>
   </si>
   <si>
-    <t>ID_OS</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>Quantidade</t>
-  </si>
-  <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 10/01/2026 </t>
   </si>
   <si>
     <t>Lucas</t>
@@ -619,9 +606,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -968,7 +954,7 @@
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.28515625" customWidth="1"/>
     <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -983,14 +969,14 @@
       <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>171</v>
+      <c r="D1" s="2" t="s">
+        <v>167</v>
       </c>
       <c r="E1" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F1" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -998,19 +984,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>900</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1018,19 +1004,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D3" s="3">
+        <v>163</v>
+      </c>
+      <c r="D3" s="2">
         <v>120</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
       </c>
       <c r="F3" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1038,19 +1024,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>168</v>
-      </c>
-      <c r="D4" s="3">
+        <v>164</v>
+      </c>
+      <c r="D4" s="2">
         <v>120</v>
       </c>
       <c r="E4" t="s">
         <v>7</v>
       </c>
       <c r="F4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1058,19 +1044,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>169</v>
-      </c>
-      <c r="D5" s="3">
+        <v>165</v>
+      </c>
+      <c r="D5" s="2">
         <v>900</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1078,19 +1064,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>170</v>
-      </c>
-      <c r="D6" s="3">
+        <v>166</v>
+      </c>
+      <c r="D6" s="2">
         <v>900</v>
       </c>
       <c r="E6" t="s">
         <v>11</v>
       </c>
       <c r="F6" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1098,19 +1084,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <v>80</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>
       </c>
       <c r="F7" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1118,19 +1104,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>167</v>
-      </c>
-      <c r="D8" s="3">
+        <v>163</v>
+      </c>
+      <c r="D8" s="2">
         <v>900</v>
       </c>
       <c r="E8" t="s">
         <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1138,19 +1124,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>168</v>
-      </c>
-      <c r="D9" s="3">
+        <v>164</v>
+      </c>
+      <c r="D9" s="2">
         <v>120</v>
       </c>
       <c r="E9" t="s">
         <v>7</v>
       </c>
       <c r="F9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1158,19 +1144,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>169</v>
-      </c>
-      <c r="D10" s="3">
+        <v>165</v>
+      </c>
+      <c r="D10" s="2">
         <v>900</v>
       </c>
       <c r="E10" t="s">
         <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1178,19 +1164,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>170</v>
-      </c>
-      <c r="D11" s="3">
+        <v>166</v>
+      </c>
+      <c r="D11" s="2">
         <v>900</v>
       </c>
       <c r="E11" t="s">
         <v>11</v>
       </c>
       <c r="F11" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1198,19 +1184,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
         <v>2</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="2">
         <v>80</v>
       </c>
       <c r="E12" t="s">
         <v>8</v>
       </c>
       <c r="F12" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1218,19 +1204,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>167</v>
-      </c>
-      <c r="D13" s="3">
+        <v>163</v>
+      </c>
+      <c r="D13" s="2">
         <v>80</v>
       </c>
       <c r="E13" t="s">
         <v>8</v>
       </c>
       <c r="F13" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1238,19 +1224,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>168</v>
-      </c>
-      <c r="D14" s="3">
+        <v>164</v>
+      </c>
+      <c r="D14" s="2">
         <v>900</v>
       </c>
       <c r="E14" t="s">
         <v>11</v>
       </c>
       <c r="F14" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1258,19 +1244,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C15" t="s">
-        <v>169</v>
-      </c>
-      <c r="D15" s="3">
+        <v>165</v>
+      </c>
+      <c r="D15" s="2">
         <v>80</v>
       </c>
       <c r="E15" t="s">
         <v>8</v>
       </c>
       <c r="F15" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1278,19 +1264,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C16" t="s">
-        <v>170</v>
-      </c>
-      <c r="D16" s="3">
+        <v>166</v>
+      </c>
+      <c r="D16" s="2">
         <v>900</v>
       </c>
       <c r="E16" t="s">
         <v>11</v>
       </c>
       <c r="F16" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1298,19 +1284,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C17" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="2">
         <v>80</v>
       </c>
       <c r="E17" t="s">
         <v>8</v>
       </c>
       <c r="F17" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1318,19 +1304,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C18" t="s">
-        <v>167</v>
-      </c>
-      <c r="D18" s="3">
+        <v>163</v>
+      </c>
+      <c r="D18" s="2">
         <v>80</v>
       </c>
       <c r="E18" t="s">
         <v>8</v>
       </c>
       <c r="F18" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1338,19 +1324,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C19" t="s">
-        <v>168</v>
-      </c>
-      <c r="D19" s="3">
+        <v>164</v>
+      </c>
+      <c r="D19" s="2">
         <v>900</v>
       </c>
       <c r="E19" t="s">
         <v>11</v>
       </c>
       <c r="F19" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1358,19 +1344,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C20" t="s">
-        <v>169</v>
-      </c>
-      <c r="D20" s="3">
+        <v>165</v>
+      </c>
+      <c r="D20" s="2">
         <v>80</v>
       </c>
       <c r="E20" t="s">
         <v>8</v>
       </c>
       <c r="F20" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1378,19 +1364,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C21" t="s">
-        <v>170</v>
-      </c>
-      <c r="D21" s="3">
+        <v>166</v>
+      </c>
+      <c r="D21" s="2">
         <v>80</v>
       </c>
       <c r="E21" t="s">
         <v>8</v>
       </c>
       <c r="F21" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1398,19 +1384,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C22" t="s">
         <v>2</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="2">
         <v>900</v>
       </c>
       <c r="E22" t="s">
         <v>11</v>
       </c>
       <c r="F22" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1418,19 +1404,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C23" t="s">
-        <v>167</v>
-      </c>
-      <c r="D23" s="3">
+        <v>163</v>
+      </c>
+      <c r="D23" s="2">
         <v>900</v>
       </c>
       <c r="E23" t="s">
         <v>11</v>
       </c>
       <c r="F23" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1438,19 +1424,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C24" t="s">
-        <v>168</v>
-      </c>
-      <c r="D24" s="3">
+        <v>164</v>
+      </c>
+      <c r="D24" s="2">
         <v>120</v>
       </c>
       <c r="E24" t="s">
         <v>7</v>
       </c>
       <c r="F24" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1458,19 +1444,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C25" t="s">
-        <v>169</v>
-      </c>
-      <c r="D25" s="3">
+        <v>165</v>
+      </c>
+      <c r="D25" s="2">
         <v>120</v>
       </c>
       <c r="E25" t="s">
         <v>7</v>
       </c>
       <c r="F25" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1478,19 +1464,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C26" t="s">
-        <v>170</v>
-      </c>
-      <c r="D26" s="3">
+        <v>166</v>
+      </c>
+      <c r="D26" s="2">
         <v>120</v>
       </c>
       <c r="E26" t="s">
         <v>7</v>
       </c>
       <c r="F26" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1498,19 +1484,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C27" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D27" s="2">
         <v>120</v>
       </c>
       <c r="E27" t="s">
         <v>7</v>
       </c>
       <c r="F27" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1518,19 +1504,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C28" t="s">
-        <v>167</v>
-      </c>
-      <c r="D28" s="3">
+        <v>163</v>
+      </c>
+      <c r="D28" s="2">
         <v>120</v>
       </c>
       <c r="E28" t="s">
         <v>7</v>
       </c>
       <c r="F28" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1538,19 +1524,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C29" t="s">
-        <v>168</v>
-      </c>
-      <c r="D29" s="3">
+        <v>164</v>
+      </c>
+      <c r="D29" s="2">
         <v>900</v>
       </c>
       <c r="E29" t="s">
         <v>11</v>
       </c>
       <c r="F29" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1558,19 +1544,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C30" t="s">
-        <v>169</v>
-      </c>
-      <c r="D30" s="3">
+        <v>165</v>
+      </c>
+      <c r="D30" s="2">
         <v>300</v>
       </c>
       <c r="E30" t="s">
         <v>9</v>
       </c>
       <c r="F30" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1578,19 +1564,19 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C31" t="s">
-        <v>170</v>
-      </c>
-      <c r="D31" s="3">
+        <v>166</v>
+      </c>
+      <c r="D31" s="2">
         <v>300</v>
       </c>
       <c r="E31" t="s">
         <v>9</v>
       </c>
       <c r="F31" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1598,19 +1584,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C32" t="s">
         <v>2</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32" s="2">
         <v>300</v>
       </c>
       <c r="E32" t="s">
         <v>9</v>
       </c>
       <c r="F32" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1618,19 +1604,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C33" t="s">
-        <v>167</v>
-      </c>
-      <c r="D33" s="3">
+        <v>163</v>
+      </c>
+      <c r="D33" s="2">
         <v>300</v>
       </c>
       <c r="E33" t="s">
         <v>9</v>
       </c>
       <c r="F33" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1638,19 +1624,19 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C34" t="s">
-        <v>168</v>
-      </c>
-      <c r="D34" s="3">
+        <v>164</v>
+      </c>
+      <c r="D34" s="2">
         <v>300</v>
       </c>
       <c r="E34" t="s">
         <v>9</v>
       </c>
       <c r="F34" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -1658,19 +1644,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C35" t="s">
-        <v>169</v>
-      </c>
-      <c r="D35" s="3">
+        <v>165</v>
+      </c>
+      <c r="D35" s="2">
         <v>900</v>
       </c>
       <c r="E35" t="s">
         <v>11</v>
       </c>
       <c r="F35" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -1678,19 +1664,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C36" t="s">
-        <v>170</v>
-      </c>
-      <c r="D36" s="3">
+        <v>166</v>
+      </c>
+      <c r="D36" s="2">
         <v>450</v>
       </c>
       <c r="E36" t="s">
         <v>10</v>
       </c>
       <c r="F36" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -1698,19 +1684,19 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C37" t="s">
         <v>2</v>
       </c>
-      <c r="D37" s="3">
+      <c r="D37" s="2">
         <v>450</v>
       </c>
       <c r="E37" t="s">
         <v>10</v>
       </c>
       <c r="F37" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -1718,19 +1704,19 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C38" t="s">
-        <v>167</v>
-      </c>
-      <c r="D38" s="3">
+        <v>163</v>
+      </c>
+      <c r="D38" s="2">
         <v>450</v>
       </c>
       <c r="E38" t="s">
         <v>10</v>
       </c>
       <c r="F38" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1738,19 +1724,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C39" t="s">
-        <v>168</v>
-      </c>
-      <c r="D39" s="3">
+        <v>164</v>
+      </c>
+      <c r="D39" s="2">
         <v>900</v>
       </c>
       <c r="E39" t="s">
         <v>11</v>
       </c>
       <c r="F39" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -1758,19 +1744,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C40" t="s">
-        <v>169</v>
-      </c>
-      <c r="D40" s="3">
+        <v>165</v>
+      </c>
+      <c r="D40" s="2">
         <v>450</v>
       </c>
       <c r="E40" t="s">
         <v>10</v>
       </c>
       <c r="F40" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -1778,19 +1764,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C41" t="s">
-        <v>170</v>
-      </c>
-      <c r="D41" s="3">
+        <v>166</v>
+      </c>
+      <c r="D41" s="2">
         <v>450</v>
       </c>
       <c r="E41" t="s">
         <v>10</v>
       </c>
       <c r="F41" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -1798,19 +1784,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C42" t="s">
         <v>2</v>
       </c>
-      <c r="D42" s="3">
+      <c r="D42" s="2">
         <v>450</v>
       </c>
       <c r="E42" t="s">
         <v>10</v>
       </c>
       <c r="F42" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -1818,19 +1804,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C43" t="s">
-        <v>167</v>
-      </c>
-      <c r="D43" s="3">
+        <v>163</v>
+      </c>
+      <c r="D43" s="2">
         <v>120</v>
       </c>
       <c r="E43" t="s">
         <v>7</v>
       </c>
       <c r="F43" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -1838,19 +1824,19 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C44" t="s">
-        <v>168</v>
-      </c>
-      <c r="D44" s="3">
+        <v>164</v>
+      </c>
+      <c r="D44" s="2">
         <v>120</v>
       </c>
       <c r="E44" t="s">
         <v>7</v>
       </c>
       <c r="F44" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -1858,19 +1844,19 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C45" t="s">
-        <v>169</v>
-      </c>
-      <c r="D45" s="3">
+        <v>165</v>
+      </c>
+      <c r="D45" s="2">
         <v>120</v>
       </c>
       <c r="E45" t="s">
         <v>7</v>
       </c>
       <c r="F45" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -1878,19 +1864,19 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C46" t="s">
-        <v>170</v>
-      </c>
-      <c r="D46" s="3">
+        <v>166</v>
+      </c>
+      <c r="D46" s="2">
         <v>120</v>
       </c>
       <c r="E46" t="s">
         <v>7</v>
       </c>
       <c r="F46" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -1898,19 +1884,19 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C47" t="s">
         <v>2</v>
       </c>
-      <c r="D47" s="3">
+      <c r="D47" s="2">
         <v>120</v>
       </c>
       <c r="E47" t="s">
         <v>7</v>
       </c>
       <c r="F47" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -1918,19 +1904,19 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C48" t="s">
-        <v>167</v>
-      </c>
-      <c r="D48" s="3">
+        <v>163</v>
+      </c>
+      <c r="D48" s="2">
         <v>120</v>
       </c>
       <c r="E48" t="s">
         <v>7</v>
       </c>
       <c r="F48" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -1938,19 +1924,19 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C49" t="s">
-        <v>168</v>
-      </c>
-      <c r="D49" s="3">
+        <v>164</v>
+      </c>
+      <c r="D49" s="2">
         <v>450</v>
       </c>
       <c r="E49" t="s">
         <v>10</v>
       </c>
       <c r="F49" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -1958,19 +1944,19 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C50" t="s">
-        <v>169</v>
-      </c>
-      <c r="D50" s="3">
+        <v>165</v>
+      </c>
+      <c r="D50" s="2">
         <v>450</v>
       </c>
       <c r="E50" t="s">
         <v>10</v>
       </c>
       <c r="F50" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -1978,19 +1964,19 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C51" t="s">
-        <v>170</v>
-      </c>
-      <c r="D51" s="3">
+        <v>166</v>
+      </c>
+      <c r="D51" s="2">
         <v>450</v>
       </c>
       <c r="E51" t="s">
         <v>10</v>
       </c>
       <c r="F51" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -1998,19 +1984,19 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C52" t="s">
         <v>2</v>
       </c>
-      <c r="D52" s="3">
+      <c r="D52" s="2">
         <v>450</v>
       </c>
       <c r="E52" t="s">
         <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -2018,19 +2004,19 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C53" t="s">
-        <v>167</v>
-      </c>
-      <c r="D53" s="3">
+        <v>163</v>
+      </c>
+      <c r="D53" s="2">
         <v>900</v>
       </c>
       <c r="E53" t="s">
         <v>11</v>
       </c>
       <c r="F53" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -2038,19 +2024,19 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C54" t="s">
-        <v>168</v>
-      </c>
-      <c r="D54" s="3">
+        <v>164</v>
+      </c>
+      <c r="D54" s="2">
         <v>450</v>
       </c>
       <c r="E54" t="s">
         <v>10</v>
       </c>
       <c r="F54" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -2058,19 +2044,19 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C55" t="s">
-        <v>169</v>
-      </c>
-      <c r="D55" s="3">
+        <v>165</v>
+      </c>
+      <c r="D55" s="2">
         <v>450</v>
       </c>
       <c r="E55" t="s">
         <v>10</v>
       </c>
       <c r="F55" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -2078,19 +2064,19 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C56" t="s">
-        <v>170</v>
-      </c>
-      <c r="D56" s="3">
+        <v>166</v>
+      </c>
+      <c r="D56" s="2">
         <v>450</v>
       </c>
       <c r="E56" t="s">
         <v>10</v>
       </c>
       <c r="F56" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -2098,19 +2084,19 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C57" t="s">
         <v>2</v>
       </c>
-      <c r="D57" s="3">
+      <c r="D57" s="2">
         <v>450</v>
       </c>
       <c r="E57" t="s">
         <v>10</v>
       </c>
       <c r="F57" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -2118,19 +2104,19 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C58" t="s">
-        <v>167</v>
-      </c>
-      <c r="D58" s="3">
+        <v>163</v>
+      </c>
+      <c r="D58" s="2">
         <v>450</v>
       </c>
       <c r="E58" t="s">
         <v>10</v>
       </c>
       <c r="F58" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -2138,19 +2124,19 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C59" t="s">
-        <v>168</v>
-      </c>
-      <c r="D59" s="3">
+        <v>164</v>
+      </c>
+      <c r="D59" s="2">
         <v>450</v>
       </c>
       <c r="E59" t="s">
         <v>10</v>
       </c>
       <c r="F59" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -2158,19 +2144,19 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C60" t="s">
-        <v>169</v>
-      </c>
-      <c r="D60" s="3">
+        <v>165</v>
+      </c>
+      <c r="D60" s="2">
         <v>450</v>
       </c>
       <c r="E60" t="s">
         <v>10</v>
       </c>
       <c r="F60" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -2178,19 +2164,19 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C61" t="s">
-        <v>170</v>
-      </c>
-      <c r="D61" s="3">
+        <v>166</v>
+      </c>
+      <c r="D61" s="2">
         <v>450</v>
       </c>
       <c r="E61" t="s">
         <v>10</v>
       </c>
       <c r="F61" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -2198,19 +2184,19 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C62" t="s">
         <v>2</v>
       </c>
-      <c r="D62" s="3">
+      <c r="D62" s="2">
         <v>900</v>
       </c>
       <c r="E62" t="s">
         <v>11</v>
       </c>
       <c r="F62" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -2218,19 +2204,19 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C63" t="s">
-        <v>167</v>
-      </c>
-      <c r="D63" s="3">
+        <v>163</v>
+      </c>
+      <c r="D63" s="2">
         <v>80</v>
       </c>
       <c r="E63" t="s">
         <v>8</v>
       </c>
       <c r="F63" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -2238,19 +2224,19 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C64" t="s">
-        <v>168</v>
-      </c>
-      <c r="D64" s="3">
+        <v>164</v>
+      </c>
+      <c r="D64" s="2">
         <v>80</v>
       </c>
       <c r="E64" t="s">
         <v>8</v>
       </c>
       <c r="F64" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -2258,19 +2244,19 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C65" t="s">
-        <v>169</v>
-      </c>
-      <c r="D65" s="3">
+        <v>165</v>
+      </c>
+      <c r="D65" s="2">
         <v>80</v>
       </c>
       <c r="E65" t="s">
         <v>8</v>
       </c>
       <c r="F65" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -2278,19 +2264,19 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C66" t="s">
-        <v>170</v>
-      </c>
-      <c r="D66" s="3">
+        <v>166</v>
+      </c>
+      <c r="D66" s="2">
         <v>120</v>
       </c>
       <c r="E66" t="s">
         <v>7</v>
       </c>
       <c r="F66" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -2298,19 +2284,19 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C67" t="s">
         <v>2</v>
       </c>
-      <c r="D67" s="3">
+      <c r="D67" s="2">
         <v>120</v>
       </c>
       <c r="E67" t="s">
         <v>7</v>
       </c>
       <c r="F67" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -2318,19 +2304,19 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C68" t="s">
-        <v>167</v>
-      </c>
-      <c r="D68" s="3">
+        <v>163</v>
+      </c>
+      <c r="D68" s="2">
         <v>120</v>
       </c>
       <c r="E68" t="s">
         <v>7</v>
       </c>
       <c r="F68" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -2338,19 +2324,19 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C69" t="s">
-        <v>168</v>
-      </c>
-      <c r="D69" s="3">
+        <v>164</v>
+      </c>
+      <c r="D69" s="2">
         <v>80</v>
       </c>
       <c r="E69" t="s">
         <v>8</v>
       </c>
       <c r="F69" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -2358,19 +2344,19 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C70" t="s">
-        <v>169</v>
-      </c>
-      <c r="D70" s="3">
+        <v>165</v>
+      </c>
+      <c r="D70" s="2">
         <v>80</v>
       </c>
       <c r="E70" t="s">
         <v>8</v>
       </c>
       <c r="F70" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -2378,19 +2364,19 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C71" t="s">
-        <v>170</v>
-      </c>
-      <c r="D71" s="3">
+        <v>166</v>
+      </c>
+      <c r="D71" s="2">
         <v>80</v>
       </c>
       <c r="E71" t="s">
         <v>8</v>
       </c>
       <c r="F71" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -2398,19 +2384,19 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C72" t="s">
         <v>2</v>
       </c>
-      <c r="D72" s="3">
+      <c r="D72" s="2">
         <v>80</v>
       </c>
       <c r="E72" t="s">
         <v>8</v>
       </c>
       <c r="F72" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -2418,19 +2404,19 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C73" t="s">
-        <v>167</v>
-      </c>
-      <c r="D73" s="3">
+        <v>163</v>
+      </c>
+      <c r="D73" s="2">
         <v>80</v>
       </c>
       <c r="E73" t="s">
         <v>8</v>
       </c>
       <c r="F73" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -2438,19 +2424,19 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C74" t="s">
-        <v>168</v>
-      </c>
-      <c r="D74" s="3">
+        <v>164</v>
+      </c>
+      <c r="D74" s="2">
         <v>80</v>
       </c>
       <c r="E74" t="s">
         <v>8</v>
       </c>
       <c r="F74" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -2458,19 +2444,19 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C75" t="s">
-        <v>169</v>
-      </c>
-      <c r="D75" s="3">
+        <v>165</v>
+      </c>
+      <c r="D75" s="2">
         <v>80</v>
       </c>
       <c r="E75" t="s">
         <v>8</v>
       </c>
       <c r="F75" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -2478,19 +2464,19 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C76" t="s">
-        <v>170</v>
-      </c>
-      <c r="D76" s="3">
+        <v>166</v>
+      </c>
+      <c r="D76" s="2">
         <v>80</v>
       </c>
       <c r="E76" t="s">
         <v>8</v>
       </c>
       <c r="F76" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -2498,19 +2484,19 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C77" t="s">
         <v>2</v>
       </c>
-      <c r="D77" s="3">
+      <c r="D77" s="2">
         <v>120</v>
       </c>
       <c r="E77" t="s">
         <v>7</v>
       </c>
       <c r="F77" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -2518,19 +2504,19 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C78" t="s">
-        <v>167</v>
-      </c>
-      <c r="D78" s="3">
+        <v>163</v>
+      </c>
+      <c r="D78" s="2">
         <v>450</v>
       </c>
       <c r="E78" t="s">
         <v>10</v>
       </c>
       <c r="F78" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -2538,19 +2524,19 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C79" t="s">
-        <v>168</v>
-      </c>
-      <c r="D79" s="3">
+        <v>164</v>
+      </c>
+      <c r="D79" s="2">
         <v>450</v>
       </c>
       <c r="E79" t="s">
         <v>10</v>
       </c>
       <c r="F79" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
@@ -2558,19 +2544,19 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C80" t="s">
-        <v>169</v>
-      </c>
-      <c r="D80" s="3">
+        <v>165</v>
+      </c>
+      <c r="D80" s="2">
         <v>450</v>
       </c>
       <c r="E80" t="s">
         <v>10</v>
       </c>
       <c r="F80" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -2578,19 +2564,19 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C81" t="s">
-        <v>170</v>
-      </c>
-      <c r="D81" s="3">
+        <v>166</v>
+      </c>
+      <c r="D81" s="2">
         <v>450</v>
       </c>
       <c r="E81" t="s">
         <v>10</v>
       </c>
       <c r="F81" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -2598,19 +2584,19 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C82" t="s">
         <v>2</v>
       </c>
-      <c r="D82" s="3">
+      <c r="D82" s="2">
         <v>450</v>
       </c>
       <c r="E82" t="s">
         <v>10</v>
       </c>
       <c r="F82" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -2618,19 +2604,19 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C83" t="s">
-        <v>167</v>
-      </c>
-      <c r="D83" s="3">
+        <v>163</v>
+      </c>
+      <c r="D83" s="2">
         <v>450</v>
       </c>
       <c r="E83" t="s">
         <v>10</v>
       </c>
       <c r="F83" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
@@ -2638,19 +2624,19 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C84" t="s">
-        <v>168</v>
-      </c>
-      <c r="D84" s="3">
+        <v>164</v>
+      </c>
+      <c r="D84" s="2">
         <v>450</v>
       </c>
       <c r="E84" t="s">
         <v>10</v>
       </c>
       <c r="F84" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
@@ -2658,19 +2644,19 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C85" t="s">
-        <v>169</v>
-      </c>
-      <c r="D85" s="3">
+        <v>165</v>
+      </c>
+      <c r="D85" s="2">
         <v>450</v>
       </c>
       <c r="E85" t="s">
         <v>10</v>
       </c>
       <c r="F85" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -2678,19 +2664,19 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C86" t="s">
-        <v>170</v>
-      </c>
-      <c r="D86" s="3">
+        <v>166</v>
+      </c>
+      <c r="D86" s="2">
         <v>450</v>
       </c>
       <c r="E86" t="s">
         <v>10</v>
       </c>
       <c r="F86" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -2698,19 +2684,19 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C87" t="s">
         <v>2</v>
       </c>
-      <c r="D87" s="3">
+      <c r="D87" s="2">
         <v>450</v>
       </c>
       <c r="E87" t="s">
         <v>10</v>
       </c>
       <c r="F87" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -2718,19 +2704,19 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C88" t="s">
-        <v>167</v>
-      </c>
-      <c r="D88" s="3">
+        <v>163</v>
+      </c>
+      <c r="D88" s="2">
         <v>450</v>
       </c>
       <c r="E88" t="s">
         <v>10</v>
       </c>
       <c r="F88" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -2738,19 +2724,19 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C89" t="s">
-        <v>168</v>
-      </c>
-      <c r="D89" s="3">
+        <v>164</v>
+      </c>
+      <c r="D89" s="2">
         <v>120</v>
       </c>
       <c r="E89" t="s">
         <v>7</v>
       </c>
       <c r="F89" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -2758,19 +2744,19 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C90" t="s">
-        <v>169</v>
-      </c>
-      <c r="D90" s="3">
+        <v>165</v>
+      </c>
+      <c r="D90" s="2">
         <v>900</v>
       </c>
       <c r="E90" t="s">
         <v>11</v>
       </c>
       <c r="F90" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
@@ -2778,19 +2764,19 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C91" t="s">
-        <v>170</v>
-      </c>
-      <c r="D91" s="3">
+        <v>166</v>
+      </c>
+      <c r="D91" s="2">
         <v>900</v>
       </c>
       <c r="E91" t="s">
         <v>11</v>
       </c>
       <c r="F91" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -2798,19 +2784,19 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C92" t="s">
         <v>2</v>
       </c>
-      <c r="D92" s="3">
+      <c r="D92" s="2">
         <v>900</v>
       </c>
       <c r="E92" t="s">
         <v>11</v>
       </c>
       <c r="F92" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -2818,19 +2804,19 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C93" t="s">
-        <v>167</v>
-      </c>
-      <c r="D93" s="3">
+        <v>163</v>
+      </c>
+      <c r="D93" s="2">
         <v>80</v>
       </c>
       <c r="E93" t="s">
         <v>8</v>
       </c>
       <c r="F93" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -2838,19 +2824,19 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C94" t="s">
-        <v>168</v>
-      </c>
-      <c r="D94" s="3">
+        <v>164</v>
+      </c>
+      <c r="D94" s="2">
         <v>900</v>
       </c>
       <c r="E94" t="s">
         <v>11</v>
       </c>
       <c r="F94" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
@@ -2858,19 +2844,19 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C95" t="s">
-        <v>169</v>
-      </c>
-      <c r="D95" s="3">
+        <v>165</v>
+      </c>
+      <c r="D95" s="2">
         <v>80</v>
       </c>
       <c r="E95" t="s">
         <v>8</v>
       </c>
       <c r="F95" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
@@ -2878,19 +2864,19 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C96" t="s">
-        <v>170</v>
-      </c>
-      <c r="D96" s="3">
+        <v>166</v>
+      </c>
+      <c r="D96" s="2">
         <v>120</v>
       </c>
       <c r="E96" t="s">
         <v>7</v>
       </c>
       <c r="F96" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -2898,19 +2884,19 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C97" t="s">
         <v>2</v>
       </c>
-      <c r="D97" s="3">
+      <c r="D97" s="2">
         <v>450</v>
       </c>
       <c r="E97" t="s">
         <v>10</v>
       </c>
       <c r="F97" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -2918,19 +2904,19 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C98" t="s">
-        <v>167</v>
-      </c>
-      <c r="D98" s="3">
+        <v>163</v>
+      </c>
+      <c r="D98" s="2">
         <v>450</v>
       </c>
       <c r="E98" t="s">
         <v>10</v>
       </c>
       <c r="F98" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -2938,19 +2924,19 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C99" t="s">
-        <v>168</v>
-      </c>
-      <c r="D99" s="3">
+        <v>164</v>
+      </c>
+      <c r="D99" s="2">
         <v>450</v>
       </c>
       <c r="E99" t="s">
         <v>10</v>
       </c>
       <c r="F99" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -2958,19 +2944,19 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C100" t="s">
-        <v>169</v>
-      </c>
-      <c r="D100" s="3">
+        <v>165</v>
+      </c>
+      <c r="D100" s="2">
         <v>450</v>
       </c>
       <c r="E100" t="s">
         <v>10</v>
       </c>
       <c r="F100" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -2978,19 +2964,19 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C101" t="s">
-        <v>170</v>
-      </c>
-      <c r="D101" s="3">
+        <v>166</v>
+      </c>
+      <c r="D101" s="2">
         <v>450</v>
       </c>
       <c r="E101" t="s">
         <v>10</v>
       </c>
       <c r="F101" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -2998,19 +2984,19 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C102" t="s">
         <v>2</v>
       </c>
-      <c r="D102" s="3">
+      <c r="D102" s="2">
         <v>450</v>
       </c>
       <c r="E102" t="s">
         <v>10</v>
       </c>
       <c r="F102" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
@@ -3018,19 +3004,19 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C103" t="s">
-        <v>167</v>
-      </c>
-      <c r="D103" s="3">
+        <v>163</v>
+      </c>
+      <c r="D103" s="2">
         <v>450</v>
       </c>
       <c r="E103" t="s">
         <v>10</v>
       </c>
       <c r="F103" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
@@ -3038,19 +3024,19 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C104" t="s">
-        <v>168</v>
-      </c>
-      <c r="D104" s="3">
+        <v>164</v>
+      </c>
+      <c r="D104" s="2">
         <v>450</v>
       </c>
       <c r="E104" t="s">
         <v>10</v>
       </c>
       <c r="F104" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
@@ -3058,19 +3044,19 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C105" t="s">
-        <v>169</v>
-      </c>
-      <c r="D105" s="3">
+        <v>165</v>
+      </c>
+      <c r="D105" s="2">
         <v>120</v>
       </c>
       <c r="E105" t="s">
         <v>7</v>
       </c>
       <c r="F105" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
@@ -3078,19 +3064,19 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C106" t="s">
-        <v>170</v>
-      </c>
-      <c r="D106" s="3">
+        <v>166</v>
+      </c>
+      <c r="D106" s="2">
         <v>80</v>
       </c>
       <c r="E106" t="s">
         <v>8</v>
       </c>
       <c r="F106" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
@@ -3098,19 +3084,19 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C107" t="s">
         <v>2</v>
       </c>
-      <c r="D107" s="3">
+      <c r="D107" s="2">
         <v>80</v>
       </c>
       <c r="E107" t="s">
         <v>8</v>
       </c>
       <c r="F107" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
@@ -3118,19 +3104,19 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C108" t="s">
-        <v>167</v>
-      </c>
-      <c r="D108" s="3">
+        <v>163</v>
+      </c>
+      <c r="D108" s="2">
         <v>80</v>
       </c>
       <c r="E108" t="s">
         <v>8</v>
       </c>
       <c r="F108" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -3138,19 +3124,19 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C109" t="s">
-        <v>168</v>
-      </c>
-      <c r="D109" s="3">
+        <v>164</v>
+      </c>
+      <c r="D109" s="2">
         <v>80</v>
       </c>
       <c r="E109" t="s">
         <v>8</v>
       </c>
       <c r="F109" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
@@ -3158,19 +3144,19 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C110" t="s">
-        <v>169</v>
-      </c>
-      <c r="D110" s="3">
+        <v>165</v>
+      </c>
+      <c r="D110" s="2">
         <v>80</v>
       </c>
       <c r="E110" t="s">
         <v>8</v>
       </c>
       <c r="F110" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -3178,19 +3164,19 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C111" t="s">
-        <v>170</v>
-      </c>
-      <c r="D111" s="3">
+        <v>166</v>
+      </c>
+      <c r="D111" s="2">
         <v>80</v>
       </c>
       <c r="E111" t="s">
         <v>8</v>
       </c>
       <c r="F111" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
@@ -3198,19 +3184,19 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C112" t="s">
         <v>2</v>
       </c>
-      <c r="D112" s="3">
+      <c r="D112" s="2">
         <v>80</v>
       </c>
       <c r="E112" t="s">
         <v>8</v>
       </c>
       <c r="F112" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
@@ -3218,19 +3204,19 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C113" t="s">
-        <v>167</v>
-      </c>
-      <c r="D113" s="3">
+        <v>163</v>
+      </c>
+      <c r="D113" s="2">
         <v>80</v>
       </c>
       <c r="E113" t="s">
         <v>8</v>
       </c>
       <c r="F113" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
@@ -3238,19 +3224,19 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C114" t="s">
-        <v>168</v>
-      </c>
-      <c r="D114" s="3">
+        <v>164</v>
+      </c>
+      <c r="D114" s="2">
         <v>900</v>
       </c>
       <c r="E114" t="s">
         <v>11</v>
       </c>
       <c r="F114" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
@@ -3258,19 +3244,19 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C115" t="s">
-        <v>169</v>
-      </c>
-      <c r="D115" s="3">
+        <v>165</v>
+      </c>
+      <c r="D115" s="2">
         <v>450</v>
       </c>
       <c r="E115" t="s">
         <v>10</v>
       </c>
       <c r="F115" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
@@ -3278,19 +3264,19 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C116" t="s">
-        <v>170</v>
-      </c>
-      <c r="D116" s="3">
+        <v>166</v>
+      </c>
+      <c r="D116" s="2">
         <v>450</v>
       </c>
       <c r="E116" t="s">
         <v>10</v>
       </c>
       <c r="F116" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
@@ -3298,19 +3284,19 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C117" t="s">
         <v>2</v>
       </c>
-      <c r="D117" s="3">
+      <c r="D117" s="2">
         <v>450</v>
       </c>
       <c r="E117" t="s">
         <v>10</v>
       </c>
       <c r="F117" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
@@ -3318,19 +3304,19 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C118" t="s">
-        <v>167</v>
-      </c>
-      <c r="D118" s="3">
+        <v>163</v>
+      </c>
+      <c r="D118" s="2">
         <v>450</v>
       </c>
       <c r="E118" t="s">
         <v>10</v>
       </c>
       <c r="F118" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
@@ -3338,19 +3324,19 @@
         <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C119" t="s">
-        <v>168</v>
-      </c>
-      <c r="D119" s="3">
+        <v>164</v>
+      </c>
+      <c r="D119" s="2">
         <v>450</v>
       </c>
       <c r="E119" t="s">
         <v>10</v>
       </c>
       <c r="F119" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
@@ -3358,19 +3344,19 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C120" t="s">
-        <v>169</v>
-      </c>
-      <c r="D120" s="3">
+        <v>165</v>
+      </c>
+      <c r="D120" s="2">
         <v>450</v>
       </c>
       <c r="E120" t="s">
         <v>10</v>
       </c>
       <c r="F120" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
@@ -3378,19 +3364,19 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C121" t="s">
-        <v>170</v>
-      </c>
-      <c r="D121" s="3">
+        <v>166</v>
+      </c>
+      <c r="D121" s="2">
         <v>450</v>
       </c>
       <c r="E121" t="s">
         <v>10</v>
       </c>
       <c r="F121" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
@@ -3398,19 +3384,19 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C122" t="s">
         <v>2</v>
       </c>
-      <c r="D122" s="3">
+      <c r="D122" s="2">
         <v>450</v>
       </c>
       <c r="E122" t="s">
         <v>10</v>
       </c>
       <c r="F122" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
@@ -3418,19 +3404,19 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C123" t="s">
-        <v>167</v>
-      </c>
-      <c r="D123" s="3">
+        <v>163</v>
+      </c>
+      <c r="D123" s="2">
         <v>450</v>
       </c>
       <c r="E123" t="s">
         <v>10</v>
       </c>
       <c r="F123" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
@@ -3438,19 +3424,19 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C124" t="s">
-        <v>168</v>
-      </c>
-      <c r="D124" s="3">
+        <v>164</v>
+      </c>
+      <c r="D124" s="2">
         <v>450</v>
       </c>
       <c r="E124" t="s">
         <v>10</v>
       </c>
       <c r="F124" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
@@ -3458,19 +3444,19 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C125" t="s">
-        <v>169</v>
-      </c>
-      <c r="D125" s="3">
+        <v>165</v>
+      </c>
+      <c r="D125" s="2">
         <v>450</v>
       </c>
       <c r="E125" t="s">
         <v>10</v>
       </c>
       <c r="F125" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
@@ -3478,19 +3464,19 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C126" t="s">
-        <v>170</v>
-      </c>
-      <c r="D126" s="3">
+        <v>166</v>
+      </c>
+      <c r="D126" s="2">
         <v>120</v>
       </c>
       <c r="E126" t="s">
         <v>7</v>
       </c>
       <c r="F126" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
@@ -3498,19 +3484,19 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C127" t="s">
         <v>2</v>
       </c>
-      <c r="D127" s="3">
+      <c r="D127" s="2">
         <v>900</v>
       </c>
       <c r="E127" t="s">
         <v>11</v>
       </c>
       <c r="F127" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
@@ -3518,19 +3504,19 @@
         <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C128" t="s">
-        <v>167</v>
-      </c>
-      <c r="D128" s="3">
+        <v>163</v>
+      </c>
+      <c r="D128" s="2">
         <v>80</v>
       </c>
       <c r="E128" t="s">
         <v>8</v>
       </c>
       <c r="F128" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
@@ -3538,19 +3524,19 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C129" t="s">
-        <v>168</v>
-      </c>
-      <c r="D129" s="3">
+        <v>164</v>
+      </c>
+      <c r="D129" s="2">
         <v>450</v>
       </c>
       <c r="E129" t="s">
         <v>10</v>
       </c>
       <c r="F129" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
@@ -3558,19 +3544,19 @@
         <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C130" t="s">
-        <v>169</v>
-      </c>
-      <c r="D130" s="3">
+        <v>165</v>
+      </c>
+      <c r="D130" s="2">
         <v>120</v>
       </c>
       <c r="E130" t="s">
         <v>7</v>
       </c>
       <c r="F130" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
@@ -3578,19 +3564,19 @@
         <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C131" t="s">
-        <v>170</v>
-      </c>
-      <c r="D131" s="3">
+        <v>166</v>
+      </c>
+      <c r="D131" s="2">
         <v>80</v>
       </c>
       <c r="E131" t="s">
         <v>8</v>
       </c>
       <c r="F131" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
@@ -3598,19 +3584,19 @@
         <v>131</v>
       </c>
       <c r="B132" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C132" t="s">
         <v>2</v>
       </c>
-      <c r="D132" s="3">
+      <c r="D132" s="2">
         <v>80</v>
       </c>
       <c r="E132" t="s">
         <v>8</v>
       </c>
       <c r="F132" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
@@ -3618,19 +3604,19 @@
         <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C133" t="s">
-        <v>167</v>
-      </c>
-      <c r="D133" s="3">
+        <v>163</v>
+      </c>
+      <c r="D133" s="2">
         <v>80</v>
       </c>
       <c r="E133" t="s">
         <v>8</v>
       </c>
       <c r="F133" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
@@ -3638,19 +3624,19 @@
         <v>133</v>
       </c>
       <c r="B134" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C134" t="s">
-        <v>168</v>
-      </c>
-      <c r="D134" s="3">
+        <v>164</v>
+      </c>
+      <c r="D134" s="2">
         <v>120</v>
       </c>
       <c r="E134" t="s">
         <v>7</v>
       </c>
       <c r="F134" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
@@ -3658,19 +3644,19 @@
         <v>134</v>
       </c>
       <c r="B135" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C135" t="s">
-        <v>169</v>
-      </c>
-      <c r="D135" s="3">
+        <v>165</v>
+      </c>
+      <c r="D135" s="2">
         <v>450</v>
       </c>
       <c r="E135" t="s">
         <v>10</v>
       </c>
       <c r="F135" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
@@ -3678,19 +3664,19 @@
         <v>135</v>
       </c>
       <c r="B136" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C136" t="s">
-        <v>170</v>
-      </c>
-      <c r="D136" s="3">
+        <v>166</v>
+      </c>
+      <c r="D136" s="2">
         <v>450</v>
       </c>
       <c r="E136" t="s">
         <v>10</v>
       </c>
       <c r="F136" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
@@ -3698,19 +3684,19 @@
         <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C137" t="s">
         <v>2</v>
       </c>
-      <c r="D137" s="3">
+      <c r="D137" s="2">
         <v>450</v>
       </c>
       <c r="E137" t="s">
         <v>10</v>
       </c>
       <c r="F137" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
@@ -3718,19 +3704,19 @@
         <v>137</v>
       </c>
       <c r="B138" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C138" t="s">
-        <v>167</v>
-      </c>
-      <c r="D138" s="3">
+        <v>163</v>
+      </c>
+      <c r="D138" s="2">
         <v>450</v>
       </c>
       <c r="E138" t="s">
         <v>10</v>
       </c>
       <c r="F138" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
@@ -3738,19 +3724,19 @@
         <v>138</v>
       </c>
       <c r="B139" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C139" t="s">
-        <v>168</v>
-      </c>
-      <c r="D139" s="3">
+        <v>164</v>
+      </c>
+      <c r="D139" s="2">
         <v>450</v>
       </c>
       <c r="E139" t="s">
         <v>10</v>
       </c>
       <c r="F139" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
@@ -3758,19 +3744,19 @@
         <v>139</v>
       </c>
       <c r="B140" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C140" t="s">
-        <v>169</v>
-      </c>
-      <c r="D140" s="3">
+        <v>165</v>
+      </c>
+      <c r="D140" s="2">
         <v>900</v>
       </c>
       <c r="E140" t="s">
         <v>11</v>
       </c>
       <c r="F140" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
@@ -3778,19 +3764,19 @@
         <v>140</v>
       </c>
       <c r="B141" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C141" t="s">
-        <v>170</v>
-      </c>
-      <c r="D141" s="3">
+        <v>166</v>
+      </c>
+      <c r="D141" s="2">
         <v>80</v>
       </c>
       <c r="E141" t="s">
         <v>8</v>
       </c>
       <c r="F141" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
@@ -3798,19 +3784,19 @@
         <v>141</v>
       </c>
       <c r="B142" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C142" t="s">
         <v>2</v>
       </c>
-      <c r="D142" s="3">
+      <c r="D142" s="2">
         <v>80</v>
       </c>
       <c r="E142" t="s">
         <v>8</v>
       </c>
       <c r="F142" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
@@ -3818,19 +3804,19 @@
         <v>142</v>
       </c>
       <c r="B143" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C143" t="s">
-        <v>167</v>
-      </c>
-      <c r="D143" s="3">
+        <v>163</v>
+      </c>
+      <c r="D143" s="2">
         <v>80</v>
       </c>
       <c r="E143" t="s">
         <v>8</v>
       </c>
       <c r="F143" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
@@ -3838,19 +3824,19 @@
         <v>143</v>
       </c>
       <c r="B144" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C144" t="s">
-        <v>168</v>
-      </c>
-      <c r="D144" s="3">
+        <v>164</v>
+      </c>
+      <c r="D144" s="2">
         <v>900</v>
       </c>
       <c r="E144" t="s">
         <v>11</v>
       </c>
       <c r="F144" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
@@ -3858,19 +3844,19 @@
         <v>144</v>
       </c>
       <c r="B145" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C145" t="s">
-        <v>169</v>
-      </c>
-      <c r="D145" s="3">
+        <v>165</v>
+      </c>
+      <c r="D145" s="2">
         <v>120</v>
       </c>
       <c r="E145" t="s">
         <v>7</v>
       </c>
       <c r="F145" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
@@ -3878,19 +3864,19 @@
         <v>145</v>
       </c>
       <c r="B146" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C146" t="s">
-        <v>170</v>
-      </c>
-      <c r="D146" s="3">
+        <v>166</v>
+      </c>
+      <c r="D146" s="2">
         <v>80</v>
       </c>
       <c r="E146" t="s">
         <v>8</v>
       </c>
       <c r="F146" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
@@ -3898,19 +3884,19 @@
         <v>146</v>
       </c>
       <c r="B147" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C147" t="s">
         <v>2</v>
       </c>
-      <c r="D147" s="3">
+      <c r="D147" s="2">
         <v>900</v>
       </c>
       <c r="E147" t="s">
         <v>11</v>
       </c>
       <c r="F147" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
@@ -3918,19 +3904,19 @@
         <v>147</v>
       </c>
       <c r="B148" t="s">
+        <v>159</v>
+      </c>
+      <c r="C148" t="s">
         <v>163</v>
       </c>
-      <c r="C148" t="s">
-        <v>167</v>
-      </c>
-      <c r="D148" s="3">
+      <c r="D148" s="2">
         <v>450</v>
       </c>
       <c r="E148" t="s">
         <v>10</v>
       </c>
       <c r="F148" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
@@ -3938,19 +3924,19 @@
         <v>148</v>
       </c>
       <c r="B149" t="s">
+        <v>160</v>
+      </c>
+      <c r="C149" t="s">
         <v>164</v>
       </c>
-      <c r="C149" t="s">
-        <v>168</v>
-      </c>
-      <c r="D149" s="3">
+      <c r="D149" s="2">
         <v>80</v>
       </c>
       <c r="E149" t="s">
         <v>8</v>
       </c>
       <c r="F149" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.25">
@@ -3958,19 +3944,19 @@
         <v>149</v>
       </c>
       <c r="B150" t="s">
+        <v>161</v>
+      </c>
+      <c r="C150" t="s">
         <v>165</v>
       </c>
-      <c r="C150" t="s">
-        <v>169</v>
-      </c>
-      <c r="D150" s="3">
+      <c r="D150" s="2">
         <v>80</v>
       </c>
       <c r="E150" t="s">
         <v>8</v>
       </c>
       <c r="F150" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
@@ -3978,19 +3964,19 @@
         <v>150</v>
       </c>
       <c r="B151" t="s">
+        <v>162</v>
+      </c>
+      <c r="C151" t="s">
         <v>166</v>
       </c>
-      <c r="C151" t="s">
-        <v>170</v>
-      </c>
-      <c r="D151" s="3">
+      <c r="D151" s="2">
         <v>80</v>
       </c>
       <c r="E151" t="s">
         <v>8</v>
       </c>
       <c r="F151" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
@@ -3998,19 +3984,19 @@
         <v>151</v>
       </c>
       <c r="B152" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C152" t="s">
         <v>2</v>
       </c>
-      <c r="D152" s="3">
+      <c r="D152" s="2">
         <v>80</v>
       </c>
       <c r="E152" t="s">
         <v>8</v>
       </c>
       <c r="F152" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
@@ -4018,26 +4004,26 @@
         <v>152</v>
       </c>
       <c r="B153" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C153" t="s">
-        <v>167</v>
-      </c>
-      <c r="D153" s="3">
+        <v>163</v>
+      </c>
+      <c r="D153" s="2">
         <v>900</v>
       </c>
       <c r="E153" t="s">
         <v>11</v>
       </c>
       <c r="F153" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A154" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D154" s="3">
+      <c r="A154" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D154" s="2">
         <f>SUM(D2:D153)</f>
         <v>55930</v>
       </c>
@@ -4125,238 +4111,4 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43212B5B-FBAB-4DDC-989A-2A4BDF07DDD2}">
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1">
-        <v>46023</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1">
-        <v>46024</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1">
-        <v>46027</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5">
-        <v>3</v>
-      </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1">
-        <v>46037</v>
-      </c>
-      <c r="C6">
-        <v>4</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1">
-        <v>46042</v>
-      </c>
-      <c r="C7">
-        <v>5</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>2</v>
-      </c>
-      <c r="F7">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1">
-        <v>46047</v>
-      </c>
-      <c r="C8">
-        <v>2</v>
-      </c>
-      <c r="D8">
-        <v>3</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1">
-        <v>46054</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9">
-        <v>5</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" s="1">
-        <v>46056</v>
-      </c>
-      <c r="C10">
-        <v>3</v>
-      </c>
-      <c r="D10">
-        <v>2</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1">
-        <v>46058</v>
-      </c>
-      <c r="C11">
-        <v>4</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
-      <c r="F11">
-        <v>120</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
 </file>
</xml_diff>